<commit_message>
Rank review sheet: collect ORCIDs from faculty pages
Every ORCID on the roster was copied from an accepted OpenAlex record, so
none is independent of the match it came from. The RA is already opening
each flagged person's faculty page for the rank check; an "ORCID (if shown)"
column costs them seconds and yields the first independently sourced
identifier we have.

The importer writes it to the person row whatever the rank decision, with a
note recording that it came from the page. If it disagrees with the ORCID
the matcher copied, the OpenAlex match is suspect: the import prints a
CONFLICT line naming the openalex_author_id to check, replaces the ORCID,
and says so in the notes. Round-tripped on the real sheet: an ORCID-only row
and a conflicting one both land correctly and touch no appointment.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/review/rank_review.xlsx
+++ b/data/review/rank_review.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use this" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Review'!$A$1:$T$140</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Review'!$A$1:$U$140</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T140"/>
+  <dimension ref="A1:U140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -502,12 +502,13 @@
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="17" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="30" customWidth="1" min="15" max="15"/>
-    <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="30" customWidth="1" min="18" max="18"/>
-    <col width="9" customWidth="1" min="19" max="19"/>
-    <col width="11" customWidth="1" min="20" max="20"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
+    <col width="30" customWidth="1" min="19" max="19"/>
+    <col width="9" customWidth="1" min="20" max="20"/>
+    <col width="11" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -583,30 +584,35 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
+          <t>ORCID (if shown)</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
           <t>Where you saw it</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Reviewed by</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>person_id</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>affiliation_id</t>
         </is>
@@ -663,16 +669,17 @@
       </c>
       <c r="M2" s="6" t="n"/>
       <c r="N2" s="6" t="n"/>
-      <c r="O2" s="7" t="n"/>
-      <c r="P2" s="6" t="n"/>
+      <c r="O2" s="6" t="n"/>
+      <c r="P2" s="7" t="n"/>
       <c r="Q2" s="6" t="n"/>
-      <c r="R2" s="7" t="n"/>
-      <c r="S2" s="3" t="inlineStr">
+      <c r="R2" s="6" t="n"/>
+      <c r="S2" s="7" t="n"/>
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="T2" s="3" t="inlineStr">
+      <c r="U2" s="3" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -729,16 +736,17 @@
       </c>
       <c r="M3" s="6" t="n"/>
       <c r="N3" s="6" t="n"/>
-      <c r="O3" s="7" t="n"/>
-      <c r="P3" s="6" t="n"/>
+      <c r="O3" s="6" t="n"/>
+      <c r="P3" s="7" t="n"/>
       <c r="Q3" s="6" t="n"/>
-      <c r="R3" s="7" t="n"/>
-      <c r="S3" s="3" t="inlineStr">
+      <c r="R3" s="6" t="n"/>
+      <c r="S3" s="7" t="n"/>
+      <c r="T3" s="3" t="inlineStr">
         <is>
           <t>169</t>
         </is>
       </c>
-      <c r="T3" s="3" t="inlineStr">
+      <c r="U3" s="3" t="inlineStr">
         <is>
           <t>170</t>
         </is>
@@ -795,16 +803,17 @@
       </c>
       <c r="M4" s="6" t="n"/>
       <c r="N4" s="6" t="n"/>
-      <c r="O4" s="7" t="n"/>
-      <c r="P4" s="6" t="n"/>
+      <c r="O4" s="6" t="n"/>
+      <c r="P4" s="7" t="n"/>
       <c r="Q4" s="6" t="n"/>
-      <c r="R4" s="7" t="n"/>
-      <c r="S4" s="3" t="inlineStr">
+      <c r="R4" s="6" t="n"/>
+      <c r="S4" s="7" t="n"/>
+      <c r="T4" s="3" t="inlineStr">
         <is>
           <t>806</t>
         </is>
       </c>
-      <c r="T4" s="3" t="inlineStr">
+      <c r="U4" s="3" t="inlineStr">
         <is>
           <t>808</t>
         </is>
@@ -861,16 +870,17 @@
       </c>
       <c r="M5" s="6" t="n"/>
       <c r="N5" s="6" t="n"/>
-      <c r="O5" s="7" t="n"/>
-      <c r="P5" s="6" t="n"/>
+      <c r="O5" s="6" t="n"/>
+      <c r="P5" s="7" t="n"/>
       <c r="Q5" s="6" t="n"/>
-      <c r="R5" s="7" t="n"/>
-      <c r="S5" s="3" t="inlineStr">
+      <c r="R5" s="6" t="n"/>
+      <c r="S5" s="7" t="n"/>
+      <c r="T5" s="3" t="inlineStr">
         <is>
           <t>797</t>
         </is>
       </c>
-      <c r="T5" s="3" t="inlineStr">
+      <c r="U5" s="3" t="inlineStr">
         <is>
           <t>798</t>
         </is>
@@ -927,16 +937,17 @@
       </c>
       <c r="M6" s="6" t="n"/>
       <c r="N6" s="6" t="n"/>
-      <c r="O6" s="7" t="n"/>
-      <c r="P6" s="6" t="n"/>
+      <c r="O6" s="6" t="n"/>
+      <c r="P6" s="7" t="n"/>
       <c r="Q6" s="6" t="n"/>
-      <c r="R6" s="7" t="n"/>
-      <c r="S6" s="3" t="inlineStr">
+      <c r="R6" s="6" t="n"/>
+      <c r="S6" s="7" t="n"/>
+      <c r="T6" s="3" t="inlineStr">
         <is>
           <t>1029</t>
         </is>
       </c>
-      <c r="T6" s="3" t="inlineStr">
+      <c r="U6" s="3" t="inlineStr">
         <is>
           <t>1031</t>
         </is>
@@ -997,16 +1008,17 @@
       </c>
       <c r="M7" s="6" t="n"/>
       <c r="N7" s="6" t="n"/>
-      <c r="O7" s="7" t="n"/>
-      <c r="P7" s="6" t="n"/>
+      <c r="O7" s="6" t="n"/>
+      <c r="P7" s="7" t="n"/>
       <c r="Q7" s="6" t="n"/>
-      <c r="R7" s="7" t="n"/>
-      <c r="S7" s="3" t="inlineStr">
+      <c r="R7" s="6" t="n"/>
+      <c r="S7" s="7" t="n"/>
+      <c r="T7" s="3" t="inlineStr">
         <is>
           <t>645</t>
         </is>
       </c>
-      <c r="T7" s="3" t="inlineStr">
+      <c r="U7" s="3" t="inlineStr">
         <is>
           <t>646</t>
         </is>
@@ -1067,16 +1079,17 @@
       </c>
       <c r="M8" s="6" t="n"/>
       <c r="N8" s="6" t="n"/>
-      <c r="O8" s="7" t="n"/>
-      <c r="P8" s="6" t="n"/>
+      <c r="O8" s="6" t="n"/>
+      <c r="P8" s="7" t="n"/>
       <c r="Q8" s="6" t="n"/>
-      <c r="R8" s="7" t="n"/>
-      <c r="S8" s="3" t="inlineStr">
+      <c r="R8" s="6" t="n"/>
+      <c r="S8" s="7" t="n"/>
+      <c r="T8" s="3" t="inlineStr">
         <is>
           <t>888</t>
         </is>
       </c>
-      <c r="T8" s="3" t="inlineStr">
+      <c r="U8" s="3" t="inlineStr">
         <is>
           <t>890</t>
         </is>
@@ -1137,16 +1150,17 @@
       </c>
       <c r="M9" s="6" t="n"/>
       <c r="N9" s="6" t="n"/>
-      <c r="O9" s="7" t="n"/>
-      <c r="P9" s="6" t="n"/>
+      <c r="O9" s="6" t="n"/>
+      <c r="P9" s="7" t="n"/>
       <c r="Q9" s="6" t="n"/>
-      <c r="R9" s="7" t="n"/>
-      <c r="S9" s="3" t="inlineStr">
+      <c r="R9" s="6" t="n"/>
+      <c r="S9" s="7" t="n"/>
+      <c r="T9" s="3" t="inlineStr">
         <is>
           <t>749</t>
         </is>
       </c>
-      <c r="T9" s="3" t="inlineStr">
+      <c r="U9" s="3" t="inlineStr">
         <is>
           <t>750</t>
         </is>
@@ -1207,16 +1221,17 @@
       </c>
       <c r="M10" s="6" t="n"/>
       <c r="N10" s="6" t="n"/>
-      <c r="O10" s="7" t="n"/>
-      <c r="P10" s="6" t="n"/>
+      <c r="O10" s="6" t="n"/>
+      <c r="P10" s="7" t="n"/>
       <c r="Q10" s="6" t="n"/>
-      <c r="R10" s="7" t="n"/>
-      <c r="S10" s="3" t="inlineStr">
+      <c r="R10" s="6" t="n"/>
+      <c r="S10" s="7" t="n"/>
+      <c r="T10" s="3" t="inlineStr">
         <is>
           <t>214</t>
         </is>
       </c>
-      <c r="T10" s="3" t="inlineStr">
+      <c r="U10" s="3" t="inlineStr">
         <is>
           <t>215</t>
         </is>
@@ -1277,16 +1292,17 @@
       </c>
       <c r="M11" s="6" t="n"/>
       <c r="N11" s="6" t="n"/>
-      <c r="O11" s="7" t="n"/>
-      <c r="P11" s="6" t="n"/>
+      <c r="O11" s="6" t="n"/>
+      <c r="P11" s="7" t="n"/>
       <c r="Q11" s="6" t="n"/>
-      <c r="R11" s="7" t="n"/>
-      <c r="S11" s="3" t="inlineStr">
+      <c r="R11" s="6" t="n"/>
+      <c r="S11" s="7" t="n"/>
+      <c r="T11" s="3" t="inlineStr">
         <is>
           <t>626</t>
         </is>
       </c>
-      <c r="T11" s="3" t="inlineStr">
+      <c r="U11" s="3" t="inlineStr">
         <is>
           <t>627</t>
         </is>
@@ -1347,16 +1363,17 @@
       </c>
       <c r="M12" s="6" t="n"/>
       <c r="N12" s="6" t="n"/>
-      <c r="O12" s="7" t="n"/>
-      <c r="P12" s="6" t="n"/>
+      <c r="O12" s="6" t="n"/>
+      <c r="P12" s="7" t="n"/>
       <c r="Q12" s="6" t="n"/>
-      <c r="R12" s="7" t="n"/>
-      <c r="S12" s="3" t="inlineStr">
+      <c r="R12" s="6" t="n"/>
+      <c r="S12" s="7" t="n"/>
+      <c r="T12" s="3" t="inlineStr">
         <is>
           <t>936</t>
         </is>
       </c>
-      <c r="T12" s="3" t="inlineStr">
+      <c r="U12" s="3" t="inlineStr">
         <is>
           <t>938</t>
         </is>
@@ -1417,16 +1434,17 @@
       </c>
       <c r="M13" s="6" t="n"/>
       <c r="N13" s="6" t="n"/>
-      <c r="O13" s="7" t="n"/>
-      <c r="P13" s="6" t="n"/>
+      <c r="O13" s="6" t="n"/>
+      <c r="P13" s="7" t="n"/>
       <c r="Q13" s="6" t="n"/>
-      <c r="R13" s="7" t="n"/>
-      <c r="S13" s="3" t="inlineStr">
+      <c r="R13" s="6" t="n"/>
+      <c r="S13" s="7" t="n"/>
+      <c r="T13" s="3" t="inlineStr">
         <is>
           <t>536</t>
         </is>
       </c>
-      <c r="T13" s="3" t="inlineStr">
+      <c r="U13" s="3" t="inlineStr">
         <is>
           <t>537</t>
         </is>
@@ -1487,16 +1505,17 @@
       </c>
       <c r="M14" s="6" t="n"/>
       <c r="N14" s="6" t="n"/>
-      <c r="O14" s="7" t="n"/>
-      <c r="P14" s="6" t="n"/>
+      <c r="O14" s="6" t="n"/>
+      <c r="P14" s="7" t="n"/>
       <c r="Q14" s="6" t="n"/>
-      <c r="R14" s="7" t="n"/>
-      <c r="S14" s="3" t="inlineStr">
+      <c r="R14" s="6" t="n"/>
+      <c r="S14" s="7" t="n"/>
+      <c r="T14" s="3" t="inlineStr">
         <is>
           <t>892</t>
         </is>
       </c>
-      <c r="T14" s="3" t="inlineStr">
+      <c r="U14" s="3" t="inlineStr">
         <is>
           <t>894</t>
         </is>
@@ -1557,16 +1576,17 @@
       </c>
       <c r="M15" s="6" t="n"/>
       <c r="N15" s="6" t="n"/>
-      <c r="O15" s="7" t="n"/>
-      <c r="P15" s="6" t="n"/>
+      <c r="O15" s="6" t="n"/>
+      <c r="P15" s="7" t="n"/>
       <c r="Q15" s="6" t="n"/>
-      <c r="R15" s="7" t="n"/>
-      <c r="S15" s="3" t="inlineStr">
+      <c r="R15" s="6" t="n"/>
+      <c r="S15" s="7" t="n"/>
+      <c r="T15" s="3" t="inlineStr">
         <is>
           <t>743</t>
         </is>
       </c>
-      <c r="T15" s="3" t="inlineStr">
+      <c r="U15" s="3" t="inlineStr">
         <is>
           <t>744</t>
         </is>
@@ -1627,16 +1647,17 @@
       </c>
       <c r="M16" s="6" t="n"/>
       <c r="N16" s="6" t="n"/>
-      <c r="O16" s="7" t="n"/>
-      <c r="P16" s="6" t="n"/>
+      <c r="O16" s="6" t="n"/>
+      <c r="P16" s="7" t="n"/>
       <c r="Q16" s="6" t="n"/>
-      <c r="R16" s="7" t="n"/>
-      <c r="S16" s="3" t="inlineStr">
+      <c r="R16" s="6" t="n"/>
+      <c r="S16" s="7" t="n"/>
+      <c r="T16" s="3" t="inlineStr">
         <is>
           <t>140</t>
         </is>
       </c>
-      <c r="T16" s="3" t="inlineStr">
+      <c r="U16" s="3" t="inlineStr">
         <is>
           <t>141</t>
         </is>
@@ -1697,16 +1718,17 @@
       </c>
       <c r="M17" s="6" t="n"/>
       <c r="N17" s="6" t="n"/>
-      <c r="O17" s="7" t="n"/>
-      <c r="P17" s="6" t="n"/>
+      <c r="O17" s="6" t="n"/>
+      <c r="P17" s="7" t="n"/>
       <c r="Q17" s="6" t="n"/>
-      <c r="R17" s="7" t="n"/>
-      <c r="S17" s="3" t="inlineStr">
+      <c r="R17" s="6" t="n"/>
+      <c r="S17" s="7" t="n"/>
+      <c r="T17" s="3" t="inlineStr">
         <is>
           <t>696</t>
         </is>
       </c>
-      <c r="T17" s="3" t="inlineStr">
+      <c r="U17" s="3" t="inlineStr">
         <is>
           <t>697</t>
         </is>
@@ -1767,16 +1789,17 @@
       </c>
       <c r="M18" s="6" t="n"/>
       <c r="N18" s="6" t="n"/>
-      <c r="O18" s="7" t="n"/>
-      <c r="P18" s="6" t="n"/>
+      <c r="O18" s="6" t="n"/>
+      <c r="P18" s="7" t="n"/>
       <c r="Q18" s="6" t="n"/>
-      <c r="R18" s="7" t="n"/>
-      <c r="S18" s="3" t="inlineStr">
+      <c r="R18" s="6" t="n"/>
+      <c r="S18" s="7" t="n"/>
+      <c r="T18" s="3" t="inlineStr">
         <is>
           <t>643</t>
         </is>
       </c>
-      <c r="T18" s="3" t="inlineStr">
+      <c r="U18" s="3" t="inlineStr">
         <is>
           <t>644</t>
         </is>
@@ -1833,16 +1856,17 @@
       </c>
       <c r="M19" s="6" t="n"/>
       <c r="N19" s="6" t="n"/>
-      <c r="O19" s="7" t="n"/>
-      <c r="P19" s="6" t="n"/>
+      <c r="O19" s="6" t="n"/>
+      <c r="P19" s="7" t="n"/>
       <c r="Q19" s="6" t="n"/>
-      <c r="R19" s="7" t="n"/>
-      <c r="S19" s="3" t="inlineStr">
+      <c r="R19" s="6" t="n"/>
+      <c r="S19" s="7" t="n"/>
+      <c r="T19" s="3" t="inlineStr">
         <is>
           <t>646</t>
         </is>
       </c>
-      <c r="T19" s="3" t="inlineStr">
+      <c r="U19" s="3" t="inlineStr">
         <is>
           <t>647</t>
         </is>
@@ -1903,16 +1927,17 @@
       </c>
       <c r="M20" s="6" t="n"/>
       <c r="N20" s="6" t="n"/>
-      <c r="O20" s="7" t="n"/>
-      <c r="P20" s="6" t="n"/>
+      <c r="O20" s="6" t="n"/>
+      <c r="P20" s="7" t="n"/>
       <c r="Q20" s="6" t="n"/>
-      <c r="R20" s="7" t="n"/>
-      <c r="S20" s="3" t="inlineStr">
+      <c r="R20" s="6" t="n"/>
+      <c r="S20" s="7" t="n"/>
+      <c r="T20" s="3" t="inlineStr">
         <is>
           <t>520</t>
         </is>
       </c>
-      <c r="T20" s="3" t="inlineStr">
+      <c r="U20" s="3" t="inlineStr">
         <is>
           <t>521</t>
         </is>
@@ -1969,16 +1994,17 @@
       </c>
       <c r="M21" s="6" t="n"/>
       <c r="N21" s="6" t="n"/>
-      <c r="O21" s="7" t="n"/>
-      <c r="P21" s="6" t="n"/>
+      <c r="O21" s="6" t="n"/>
+      <c r="P21" s="7" t="n"/>
       <c r="Q21" s="6" t="n"/>
-      <c r="R21" s="7" t="n"/>
-      <c r="S21" s="3" t="inlineStr">
+      <c r="R21" s="6" t="n"/>
+      <c r="S21" s="7" t="n"/>
+      <c r="T21" s="3" t="inlineStr">
         <is>
           <t>374</t>
         </is>
       </c>
-      <c r="T21" s="3" t="inlineStr">
+      <c r="U21" s="3" t="inlineStr">
         <is>
           <t>375</t>
         </is>
@@ -2035,16 +2061,17 @@
       </c>
       <c r="M22" s="6" t="n"/>
       <c r="N22" s="6" t="n"/>
-      <c r="O22" s="7" t="n"/>
-      <c r="P22" s="6" t="n"/>
+      <c r="O22" s="6" t="n"/>
+      <c r="P22" s="7" t="n"/>
       <c r="Q22" s="6" t="n"/>
-      <c r="R22" s="7" t="n"/>
-      <c r="S22" s="3" t="inlineStr">
+      <c r="R22" s="6" t="n"/>
+      <c r="S22" s="7" t="n"/>
+      <c r="T22" s="3" t="inlineStr">
         <is>
           <t>878</t>
         </is>
       </c>
-      <c r="T22" s="3" t="inlineStr">
+      <c r="U22" s="3" t="inlineStr">
         <is>
           <t>880</t>
         </is>
@@ -2105,16 +2132,17 @@
       </c>
       <c r="M23" s="6" t="n"/>
       <c r="N23" s="6" t="n"/>
-      <c r="O23" s="7" t="n"/>
-      <c r="P23" s="6" t="n"/>
+      <c r="O23" s="6" t="n"/>
+      <c r="P23" s="7" t="n"/>
       <c r="Q23" s="6" t="n"/>
-      <c r="R23" s="7" t="n"/>
-      <c r="S23" s="3" t="inlineStr">
+      <c r="R23" s="6" t="n"/>
+      <c r="S23" s="7" t="n"/>
+      <c r="T23" s="3" t="inlineStr">
         <is>
           <t>541</t>
         </is>
       </c>
-      <c r="T23" s="3" t="inlineStr">
+      <c r="U23" s="3" t="inlineStr">
         <is>
           <t>542</t>
         </is>
@@ -2175,16 +2203,17 @@
       </c>
       <c r="M24" s="6" t="n"/>
       <c r="N24" s="6" t="n"/>
-      <c r="O24" s="7" t="n"/>
-      <c r="P24" s="6" t="n"/>
+      <c r="O24" s="6" t="n"/>
+      <c r="P24" s="7" t="n"/>
       <c r="Q24" s="6" t="n"/>
-      <c r="R24" s="7" t="n"/>
-      <c r="S24" s="3" t="inlineStr">
+      <c r="R24" s="6" t="n"/>
+      <c r="S24" s="7" t="n"/>
+      <c r="T24" s="3" t="inlineStr">
         <is>
           <t>243</t>
         </is>
       </c>
-      <c r="T24" s="3" t="inlineStr">
+      <c r="U24" s="3" t="inlineStr">
         <is>
           <t>244</t>
         </is>
@@ -2245,16 +2274,17 @@
       </c>
       <c r="M25" s="6" t="n"/>
       <c r="N25" s="6" t="n"/>
-      <c r="O25" s="7" t="n"/>
-      <c r="P25" s="6" t="n"/>
+      <c r="O25" s="6" t="n"/>
+      <c r="P25" s="7" t="n"/>
       <c r="Q25" s="6" t="n"/>
-      <c r="R25" s="7" t="n"/>
-      <c r="S25" s="3" t="inlineStr">
+      <c r="R25" s="6" t="n"/>
+      <c r="S25" s="7" t="n"/>
+      <c r="T25" s="3" t="inlineStr">
         <is>
           <t>945</t>
         </is>
       </c>
-      <c r="T25" s="3" t="inlineStr">
+      <c r="U25" s="3" t="inlineStr">
         <is>
           <t>947</t>
         </is>
@@ -2315,16 +2345,17 @@
       </c>
       <c r="M26" s="6" t="n"/>
       <c r="N26" s="6" t="n"/>
-      <c r="O26" s="7" t="n"/>
-      <c r="P26" s="6" t="n"/>
+      <c r="O26" s="6" t="n"/>
+      <c r="P26" s="7" t="n"/>
       <c r="Q26" s="6" t="n"/>
-      <c r="R26" s="7" t="n"/>
-      <c r="S26" s="3" t="inlineStr">
+      <c r="R26" s="6" t="n"/>
+      <c r="S26" s="7" t="n"/>
+      <c r="T26" s="3" t="inlineStr">
         <is>
           <t>91</t>
         </is>
       </c>
-      <c r="T26" s="3" t="inlineStr">
+      <c r="U26" s="3" t="inlineStr">
         <is>
           <t>92</t>
         </is>
@@ -2385,16 +2416,17 @@
       </c>
       <c r="M27" s="6" t="n"/>
       <c r="N27" s="6" t="n"/>
-      <c r="O27" s="7" t="n"/>
-      <c r="P27" s="6" t="n"/>
+      <c r="O27" s="6" t="n"/>
+      <c r="P27" s="7" t="n"/>
       <c r="Q27" s="6" t="n"/>
-      <c r="R27" s="7" t="n"/>
-      <c r="S27" s="3" t="inlineStr">
+      <c r="R27" s="6" t="n"/>
+      <c r="S27" s="7" t="n"/>
+      <c r="T27" s="3" t="inlineStr">
         <is>
           <t>954</t>
         </is>
       </c>
-      <c r="T27" s="3" t="inlineStr">
+      <c r="U27" s="3" t="inlineStr">
         <is>
           <t>956</t>
         </is>
@@ -2451,16 +2483,17 @@
       </c>
       <c r="M28" s="6" t="n"/>
       <c r="N28" s="6" t="n"/>
-      <c r="O28" s="7" t="n"/>
-      <c r="P28" s="6" t="n"/>
+      <c r="O28" s="6" t="n"/>
+      <c r="P28" s="7" t="n"/>
       <c r="Q28" s="6" t="n"/>
-      <c r="R28" s="7" t="n"/>
-      <c r="S28" s="3" t="inlineStr">
+      <c r="R28" s="6" t="n"/>
+      <c r="S28" s="7" t="n"/>
+      <c r="T28" s="3" t="inlineStr">
         <is>
           <t>702</t>
         </is>
       </c>
-      <c r="T28" s="3" t="inlineStr">
+      <c r="U28" s="3" t="inlineStr">
         <is>
           <t>703</t>
         </is>
@@ -2521,16 +2554,17 @@
       </c>
       <c r="M29" s="6" t="n"/>
       <c r="N29" s="6" t="n"/>
-      <c r="O29" s="7" t="n"/>
-      <c r="P29" s="6" t="n"/>
+      <c r="O29" s="6" t="n"/>
+      <c r="P29" s="7" t="n"/>
       <c r="Q29" s="6" t="n"/>
-      <c r="R29" s="7" t="n"/>
-      <c r="S29" s="3" t="inlineStr">
+      <c r="R29" s="6" t="n"/>
+      <c r="S29" s="7" t="n"/>
+      <c r="T29" s="3" t="inlineStr">
         <is>
           <t>624</t>
         </is>
       </c>
-      <c r="T29" s="3" t="inlineStr">
+      <c r="U29" s="3" t="inlineStr">
         <is>
           <t>625</t>
         </is>
@@ -2591,16 +2625,17 @@
       </c>
       <c r="M30" s="12" t="n"/>
       <c r="N30" s="12" t="n"/>
-      <c r="O30" s="13" t="n"/>
-      <c r="P30" s="12" t="n"/>
+      <c r="O30" s="12" t="n"/>
+      <c r="P30" s="13" t="n"/>
       <c r="Q30" s="12" t="n"/>
-      <c r="R30" s="13" t="n"/>
-      <c r="S30" s="9" t="inlineStr">
+      <c r="R30" s="12" t="n"/>
+      <c r="S30" s="13" t="n"/>
+      <c r="T30" s="9" t="inlineStr">
         <is>
           <t>373</t>
         </is>
       </c>
-      <c r="T30" s="9" t="inlineStr">
+      <c r="U30" s="9" t="inlineStr">
         <is>
           <t>374</t>
         </is>
@@ -2657,16 +2692,17 @@
       </c>
       <c r="M31" s="6" t="n"/>
       <c r="N31" s="6" t="n"/>
-      <c r="O31" s="7" t="n"/>
-      <c r="P31" s="6" t="n"/>
+      <c r="O31" s="6" t="n"/>
+      <c r="P31" s="7" t="n"/>
       <c r="Q31" s="6" t="n"/>
-      <c r="R31" s="7" t="n"/>
-      <c r="S31" s="3" t="inlineStr">
+      <c r="R31" s="6" t="n"/>
+      <c r="S31" s="7" t="n"/>
+      <c r="T31" s="3" t="inlineStr">
         <is>
           <t>773</t>
         </is>
       </c>
-      <c r="T31" s="3" t="inlineStr">
+      <c r="U31" s="3" t="inlineStr">
         <is>
           <t>774</t>
         </is>
@@ -2727,16 +2763,17 @@
       </c>
       <c r="M32" s="6" t="n"/>
       <c r="N32" s="6" t="n"/>
-      <c r="O32" s="7" t="n"/>
-      <c r="P32" s="6" t="n"/>
+      <c r="O32" s="6" t="n"/>
+      <c r="P32" s="7" t="n"/>
       <c r="Q32" s="6" t="n"/>
-      <c r="R32" s="7" t="n"/>
-      <c r="S32" s="3" t="inlineStr">
+      <c r="R32" s="6" t="n"/>
+      <c r="S32" s="7" t="n"/>
+      <c r="T32" s="3" t="inlineStr">
         <is>
           <t>222</t>
         </is>
       </c>
-      <c r="T32" s="3" t="inlineStr">
+      <c r="U32" s="3" t="inlineStr">
         <is>
           <t>223</t>
         </is>
@@ -2797,16 +2834,17 @@
       </c>
       <c r="M33" s="6" t="n"/>
       <c r="N33" s="6" t="n"/>
-      <c r="O33" s="7" t="n"/>
-      <c r="P33" s="6" t="n"/>
+      <c r="O33" s="6" t="n"/>
+      <c r="P33" s="7" t="n"/>
       <c r="Q33" s="6" t="n"/>
-      <c r="R33" s="7" t="n"/>
-      <c r="S33" s="3" t="inlineStr">
+      <c r="R33" s="6" t="n"/>
+      <c r="S33" s="7" t="n"/>
+      <c r="T33" s="3" t="inlineStr">
         <is>
           <t>210</t>
         </is>
       </c>
-      <c r="T33" s="3" t="inlineStr">
+      <c r="U33" s="3" t="inlineStr">
         <is>
           <t>211</t>
         </is>
@@ -2867,16 +2905,17 @@
       </c>
       <c r="M34" s="6" t="n"/>
       <c r="N34" s="6" t="n"/>
-      <c r="O34" s="7" t="n"/>
-      <c r="P34" s="6" t="n"/>
+      <c r="O34" s="6" t="n"/>
+      <c r="P34" s="7" t="n"/>
       <c r="Q34" s="6" t="n"/>
-      <c r="R34" s="7" t="n"/>
-      <c r="S34" s="3" t="inlineStr">
+      <c r="R34" s="6" t="n"/>
+      <c r="S34" s="7" t="n"/>
+      <c r="T34" s="3" t="inlineStr">
         <is>
           <t>539</t>
         </is>
       </c>
-      <c r="T34" s="3" t="inlineStr">
+      <c r="U34" s="3" t="inlineStr">
         <is>
           <t>540</t>
         </is>
@@ -2933,16 +2972,17 @@
       </c>
       <c r="M35" s="6" t="n"/>
       <c r="N35" s="6" t="n"/>
-      <c r="O35" s="7" t="n"/>
-      <c r="P35" s="6" t="n"/>
+      <c r="O35" s="6" t="n"/>
+      <c r="P35" s="7" t="n"/>
       <c r="Q35" s="6" t="n"/>
-      <c r="R35" s="7" t="n"/>
-      <c r="S35" s="3" t="inlineStr">
+      <c r="R35" s="6" t="n"/>
+      <c r="S35" s="7" t="n"/>
+      <c r="T35" s="3" t="inlineStr">
         <is>
           <t>49</t>
         </is>
       </c>
-      <c r="T35" s="3" t="inlineStr">
+      <c r="U35" s="3" t="inlineStr">
         <is>
           <t>49</t>
         </is>
@@ -3003,16 +3043,17 @@
       </c>
       <c r="M36" s="6" t="n"/>
       <c r="N36" s="6" t="n"/>
-      <c r="O36" s="7" t="n"/>
-      <c r="P36" s="6" t="n"/>
+      <c r="O36" s="6" t="n"/>
+      <c r="P36" s="7" t="n"/>
       <c r="Q36" s="6" t="n"/>
-      <c r="R36" s="7" t="n"/>
-      <c r="S36" s="3" t="inlineStr">
+      <c r="R36" s="6" t="n"/>
+      <c r="S36" s="7" t="n"/>
+      <c r="T36" s="3" t="inlineStr">
         <is>
           <t>655</t>
         </is>
       </c>
-      <c r="T36" s="3" t="inlineStr">
+      <c r="U36" s="3" t="inlineStr">
         <is>
           <t>656</t>
         </is>
@@ -3073,16 +3114,17 @@
       </c>
       <c r="M37" s="6" t="n"/>
       <c r="N37" s="6" t="n"/>
-      <c r="O37" s="7" t="n"/>
-      <c r="P37" s="6" t="n"/>
+      <c r="O37" s="6" t="n"/>
+      <c r="P37" s="7" t="n"/>
       <c r="Q37" s="6" t="n"/>
-      <c r="R37" s="7" t="n"/>
-      <c r="S37" s="3" t="inlineStr">
+      <c r="R37" s="6" t="n"/>
+      <c r="S37" s="7" t="n"/>
+      <c r="T37" s="3" t="inlineStr">
         <is>
           <t>832</t>
         </is>
       </c>
-      <c r="T37" s="3" t="inlineStr">
+      <c r="U37" s="3" t="inlineStr">
         <is>
           <t>834</t>
         </is>
@@ -3143,16 +3185,17 @@
       </c>
       <c r="M38" s="6" t="n"/>
       <c r="N38" s="6" t="n"/>
-      <c r="O38" s="7" t="n"/>
-      <c r="P38" s="6" t="n"/>
+      <c r="O38" s="6" t="n"/>
+      <c r="P38" s="7" t="n"/>
       <c r="Q38" s="6" t="n"/>
-      <c r="R38" s="7" t="n"/>
-      <c r="S38" s="3" t="inlineStr">
+      <c r="R38" s="6" t="n"/>
+      <c r="S38" s="7" t="n"/>
+      <c r="T38" s="3" t="inlineStr">
         <is>
           <t>127</t>
         </is>
       </c>
-      <c r="T38" s="3" t="inlineStr">
+      <c r="U38" s="3" t="inlineStr">
         <is>
           <t>128</t>
         </is>
@@ -3209,16 +3252,17 @@
       </c>
       <c r="M39" s="6" t="n"/>
       <c r="N39" s="6" t="n"/>
-      <c r="O39" s="7" t="n"/>
-      <c r="P39" s="6" t="n"/>
+      <c r="O39" s="6" t="n"/>
+      <c r="P39" s="7" t="n"/>
       <c r="Q39" s="6" t="n"/>
-      <c r="R39" s="7" t="n"/>
-      <c r="S39" s="3" t="inlineStr">
+      <c r="R39" s="6" t="n"/>
+      <c r="S39" s="7" t="n"/>
+      <c r="T39" s="3" t="inlineStr">
         <is>
           <t>1035</t>
         </is>
       </c>
-      <c r="T39" s="3" t="inlineStr">
+      <c r="U39" s="3" t="inlineStr">
         <is>
           <t>1037</t>
         </is>
@@ -3279,16 +3323,17 @@
       </c>
       <c r="M40" s="6" t="n"/>
       <c r="N40" s="6" t="n"/>
-      <c r="O40" s="7" t="n"/>
-      <c r="P40" s="6" t="n"/>
+      <c r="O40" s="6" t="n"/>
+      <c r="P40" s="7" t="n"/>
       <c r="Q40" s="6" t="n"/>
-      <c r="R40" s="7" t="n"/>
-      <c r="S40" s="3" t="inlineStr">
+      <c r="R40" s="6" t="n"/>
+      <c r="S40" s="7" t="n"/>
+      <c r="T40" s="3" t="inlineStr">
         <is>
           <t>519</t>
         </is>
       </c>
-      <c r="T40" s="3" t="inlineStr">
+      <c r="U40" s="3" t="inlineStr">
         <is>
           <t>520</t>
         </is>
@@ -3349,16 +3394,17 @@
       </c>
       <c r="M41" s="6" t="n"/>
       <c r="N41" s="6" t="n"/>
-      <c r="O41" s="7" t="n"/>
-      <c r="P41" s="6" t="n"/>
+      <c r="O41" s="6" t="n"/>
+      <c r="P41" s="7" t="n"/>
       <c r="Q41" s="6" t="n"/>
-      <c r="R41" s="7" t="n"/>
-      <c r="S41" s="3" t="inlineStr">
+      <c r="R41" s="6" t="n"/>
+      <c r="S41" s="7" t="n"/>
+      <c r="T41" s="3" t="inlineStr">
         <is>
           <t>554</t>
         </is>
       </c>
-      <c r="T41" s="3" t="inlineStr">
+      <c r="U41" s="3" t="inlineStr">
         <is>
           <t>555</t>
         </is>
@@ -3419,16 +3465,17 @@
       </c>
       <c r="M42" s="6" t="n"/>
       <c r="N42" s="6" t="n"/>
-      <c r="O42" s="7" t="n"/>
-      <c r="P42" s="6" t="n"/>
+      <c r="O42" s="6" t="n"/>
+      <c r="P42" s="7" t="n"/>
       <c r="Q42" s="6" t="n"/>
-      <c r="R42" s="7" t="n"/>
-      <c r="S42" s="3" t="inlineStr">
+      <c r="R42" s="6" t="n"/>
+      <c r="S42" s="7" t="n"/>
+      <c r="T42" s="3" t="inlineStr">
         <is>
           <t>215</t>
         </is>
       </c>
-      <c r="T42" s="3" t="inlineStr">
+      <c r="U42" s="3" t="inlineStr">
         <is>
           <t>216</t>
         </is>
@@ -3489,16 +3536,17 @@
       </c>
       <c r="M43" s="6" t="n"/>
       <c r="N43" s="6" t="n"/>
-      <c r="O43" s="7" t="n"/>
-      <c r="P43" s="6" t="n"/>
+      <c r="O43" s="6" t="n"/>
+      <c r="P43" s="7" t="n"/>
       <c r="Q43" s="6" t="n"/>
-      <c r="R43" s="7" t="n"/>
-      <c r="S43" s="3" t="inlineStr">
+      <c r="R43" s="6" t="n"/>
+      <c r="S43" s="7" t="n"/>
+      <c r="T43" s="3" t="inlineStr">
         <is>
           <t>427</t>
         </is>
       </c>
-      <c r="T43" s="3" t="inlineStr">
+      <c r="U43" s="3" t="inlineStr">
         <is>
           <t>428</t>
         </is>
@@ -3555,16 +3603,17 @@
       </c>
       <c r="M44" s="6" t="n"/>
       <c r="N44" s="6" t="n"/>
-      <c r="O44" s="7" t="n"/>
-      <c r="P44" s="6" t="n"/>
+      <c r="O44" s="6" t="n"/>
+      <c r="P44" s="7" t="n"/>
       <c r="Q44" s="6" t="n"/>
-      <c r="R44" s="7" t="n"/>
-      <c r="S44" s="3" t="inlineStr">
+      <c r="R44" s="6" t="n"/>
+      <c r="S44" s="7" t="n"/>
+      <c r="T44" s="3" t="inlineStr">
         <is>
           <t>613</t>
         </is>
       </c>
-      <c r="T44" s="3" t="inlineStr">
+      <c r="U44" s="3" t="inlineStr">
         <is>
           <t>614</t>
         </is>
@@ -3625,16 +3674,17 @@
       </c>
       <c r="M45" s="6" t="n"/>
       <c r="N45" s="6" t="n"/>
-      <c r="O45" s="7" t="n"/>
-      <c r="P45" s="6" t="n"/>
+      <c r="O45" s="6" t="n"/>
+      <c r="P45" s="7" t="n"/>
       <c r="Q45" s="6" t="n"/>
-      <c r="R45" s="7" t="n"/>
-      <c r="S45" s="3" t="inlineStr">
+      <c r="R45" s="6" t="n"/>
+      <c r="S45" s="7" t="n"/>
+      <c r="T45" s="3" t="inlineStr">
         <is>
           <t>944</t>
         </is>
       </c>
-      <c r="T45" s="3" t="inlineStr">
+      <c r="U45" s="3" t="inlineStr">
         <is>
           <t>946</t>
         </is>
@@ -3695,16 +3745,17 @@
       </c>
       <c r="M46" s="6" t="n"/>
       <c r="N46" s="6" t="n"/>
-      <c r="O46" s="7" t="n"/>
-      <c r="P46" s="6" t="n"/>
+      <c r="O46" s="6" t="n"/>
+      <c r="P46" s="7" t="n"/>
       <c r="Q46" s="6" t="n"/>
-      <c r="R46" s="7" t="n"/>
-      <c r="S46" s="3" t="inlineStr">
+      <c r="R46" s="6" t="n"/>
+      <c r="S46" s="7" t="n"/>
+      <c r="T46" s="3" t="inlineStr">
         <is>
           <t>649</t>
         </is>
       </c>
-      <c r="T46" s="3" t="inlineStr">
+      <c r="U46" s="3" t="inlineStr">
         <is>
           <t>650</t>
         </is>
@@ -3765,16 +3816,17 @@
       </c>
       <c r="M47" s="6" t="n"/>
       <c r="N47" s="6" t="n"/>
-      <c r="O47" s="7" t="n"/>
-      <c r="P47" s="6" t="n"/>
+      <c r="O47" s="6" t="n"/>
+      <c r="P47" s="7" t="n"/>
       <c r="Q47" s="6" t="n"/>
-      <c r="R47" s="7" t="n"/>
-      <c r="S47" s="3" t="inlineStr">
+      <c r="R47" s="6" t="n"/>
+      <c r="S47" s="7" t="n"/>
+      <c r="T47" s="3" t="inlineStr">
         <is>
           <t>972</t>
         </is>
       </c>
-      <c r="T47" s="3" t="inlineStr">
+      <c r="U47" s="3" t="inlineStr">
         <is>
           <t>974</t>
         </is>
@@ -3831,16 +3883,17 @@
       </c>
       <c r="M48" s="6" t="n"/>
       <c r="N48" s="6" t="n"/>
-      <c r="O48" s="7" t="n"/>
-      <c r="P48" s="6" t="n"/>
+      <c r="O48" s="6" t="n"/>
+      <c r="P48" s="7" t="n"/>
       <c r="Q48" s="6" t="n"/>
-      <c r="R48" s="7" t="n"/>
-      <c r="S48" s="3" t="inlineStr">
+      <c r="R48" s="6" t="n"/>
+      <c r="S48" s="7" t="n"/>
+      <c r="T48" s="3" t="inlineStr">
         <is>
           <t>678</t>
         </is>
       </c>
-      <c r="T48" s="3" t="inlineStr">
+      <c r="U48" s="3" t="inlineStr">
         <is>
           <t>679</t>
         </is>
@@ -3901,16 +3954,17 @@
       </c>
       <c r="M49" s="6" t="n"/>
       <c r="N49" s="6" t="n"/>
-      <c r="O49" s="7" t="n"/>
-      <c r="P49" s="6" t="n"/>
+      <c r="O49" s="6" t="n"/>
+      <c r="P49" s="7" t="n"/>
       <c r="Q49" s="6" t="n"/>
-      <c r="R49" s="7" t="n"/>
-      <c r="S49" s="3" t="inlineStr">
+      <c r="R49" s="6" t="n"/>
+      <c r="S49" s="7" t="n"/>
+      <c r="T49" s="3" t="inlineStr">
         <is>
           <t>661</t>
         </is>
       </c>
-      <c r="T49" s="3" t="inlineStr">
+      <c r="U49" s="3" t="inlineStr">
         <is>
           <t>662</t>
         </is>
@@ -3971,16 +4025,17 @@
       </c>
       <c r="M50" s="6" t="n"/>
       <c r="N50" s="6" t="n"/>
-      <c r="O50" s="7" t="n"/>
-      <c r="P50" s="6" t="n"/>
+      <c r="O50" s="6" t="n"/>
+      <c r="P50" s="7" t="n"/>
       <c r="Q50" s="6" t="n"/>
-      <c r="R50" s="7" t="n"/>
-      <c r="S50" s="3" t="inlineStr">
+      <c r="R50" s="6" t="n"/>
+      <c r="S50" s="7" t="n"/>
+      <c r="T50" s="3" t="inlineStr">
         <is>
           <t>654</t>
         </is>
       </c>
-      <c r="T50" s="3" t="inlineStr">
+      <c r="U50" s="3" t="inlineStr">
         <is>
           <t>655</t>
         </is>
@@ -4041,16 +4096,17 @@
       </c>
       <c r="M51" s="6" t="n"/>
       <c r="N51" s="6" t="n"/>
-      <c r="O51" s="7" t="n"/>
-      <c r="P51" s="6" t="n"/>
+      <c r="O51" s="6" t="n"/>
+      <c r="P51" s="7" t="n"/>
       <c r="Q51" s="6" t="n"/>
-      <c r="R51" s="7" t="n"/>
-      <c r="S51" s="3" t="inlineStr">
+      <c r="R51" s="6" t="n"/>
+      <c r="S51" s="7" t="n"/>
+      <c r="T51" s="3" t="inlineStr">
         <is>
           <t>869</t>
         </is>
       </c>
-      <c r="T51" s="3" t="inlineStr">
+      <c r="U51" s="3" t="inlineStr">
         <is>
           <t>871</t>
         </is>
@@ -4107,16 +4163,17 @@
       </c>
       <c r="M52" s="6" t="n"/>
       <c r="N52" s="6" t="n"/>
-      <c r="O52" s="7" t="n"/>
-      <c r="P52" s="6" t="n"/>
+      <c r="O52" s="6" t="n"/>
+      <c r="P52" s="7" t="n"/>
       <c r="Q52" s="6" t="n"/>
-      <c r="R52" s="7" t="n"/>
-      <c r="S52" s="3" t="inlineStr">
+      <c r="R52" s="6" t="n"/>
+      <c r="S52" s="7" t="n"/>
+      <c r="T52" s="3" t="inlineStr">
         <is>
           <t>451</t>
         </is>
       </c>
-      <c r="T52" s="3" t="inlineStr">
+      <c r="U52" s="3" t="inlineStr">
         <is>
           <t>452</t>
         </is>
@@ -4173,16 +4230,17 @@
       </c>
       <c r="M53" s="6" t="n"/>
       <c r="N53" s="6" t="n"/>
-      <c r="O53" s="7" t="n"/>
-      <c r="P53" s="6" t="n"/>
+      <c r="O53" s="6" t="n"/>
+      <c r="P53" s="7" t="n"/>
       <c r="Q53" s="6" t="n"/>
-      <c r="R53" s="7" t="n"/>
-      <c r="S53" s="3" t="inlineStr">
+      <c r="R53" s="6" t="n"/>
+      <c r="S53" s="7" t="n"/>
+      <c r="T53" s="3" t="inlineStr">
         <is>
           <t>34</t>
         </is>
       </c>
-      <c r="T53" s="3" t="inlineStr">
+      <c r="U53" s="3" t="inlineStr">
         <is>
           <t>34</t>
         </is>
@@ -4239,16 +4297,17 @@
       </c>
       <c r="M54" s="6" t="n"/>
       <c r="N54" s="6" t="n"/>
-      <c r="O54" s="7" t="n"/>
-      <c r="P54" s="6" t="n"/>
+      <c r="O54" s="6" t="n"/>
+      <c r="P54" s="7" t="n"/>
       <c r="Q54" s="6" t="n"/>
-      <c r="R54" s="7" t="n"/>
-      <c r="S54" s="3" t="inlineStr">
+      <c r="R54" s="6" t="n"/>
+      <c r="S54" s="7" t="n"/>
+      <c r="T54" s="3" t="inlineStr">
         <is>
           <t>474</t>
         </is>
       </c>
-      <c r="T54" s="3" t="inlineStr">
+      <c r="U54" s="3" t="inlineStr">
         <is>
           <t>475</t>
         </is>
@@ -4309,16 +4368,17 @@
       </c>
       <c r="M55" s="6" t="n"/>
       <c r="N55" s="6" t="n"/>
-      <c r="O55" s="7" t="n"/>
-      <c r="P55" s="6" t="n"/>
+      <c r="O55" s="6" t="n"/>
+      <c r="P55" s="7" t="n"/>
       <c r="Q55" s="6" t="n"/>
-      <c r="R55" s="7" t="n"/>
-      <c r="S55" s="3" t="inlineStr">
+      <c r="R55" s="6" t="n"/>
+      <c r="S55" s="7" t="n"/>
+      <c r="T55" s="3" t="inlineStr">
         <is>
           <t>805</t>
         </is>
       </c>
-      <c r="T55" s="3" t="inlineStr">
+      <c r="U55" s="3" t="inlineStr">
         <is>
           <t>807</t>
         </is>
@@ -4375,16 +4435,17 @@
       </c>
       <c r="M56" s="6" t="n"/>
       <c r="N56" s="6" t="n"/>
-      <c r="O56" s="7" t="n"/>
-      <c r="P56" s="6" t="n"/>
+      <c r="O56" s="6" t="n"/>
+      <c r="P56" s="7" t="n"/>
       <c r="Q56" s="6" t="n"/>
-      <c r="R56" s="7" t="n"/>
-      <c r="S56" s="3" t="inlineStr">
+      <c r="R56" s="6" t="n"/>
+      <c r="S56" s="7" t="n"/>
+      <c r="T56" s="3" t="inlineStr">
         <is>
           <t>1037</t>
         </is>
       </c>
-      <c r="T56" s="3" t="inlineStr">
+      <c r="U56" s="3" t="inlineStr">
         <is>
           <t>1039</t>
         </is>
@@ -4445,16 +4506,17 @@
       </c>
       <c r="M57" s="6" t="n"/>
       <c r="N57" s="6" t="n"/>
-      <c r="O57" s="7" t="n"/>
-      <c r="P57" s="6" t="n"/>
+      <c r="O57" s="6" t="n"/>
+      <c r="P57" s="7" t="n"/>
       <c r="Q57" s="6" t="n"/>
-      <c r="R57" s="7" t="n"/>
-      <c r="S57" s="3" t="inlineStr">
+      <c r="R57" s="6" t="n"/>
+      <c r="S57" s="7" t="n"/>
+      <c r="T57" s="3" t="inlineStr">
         <is>
           <t>424</t>
         </is>
       </c>
-      <c r="T57" s="3" t="inlineStr">
+      <c r="U57" s="3" t="inlineStr">
         <is>
           <t>425</t>
         </is>
@@ -4515,16 +4577,17 @@
       </c>
       <c r="M58" s="6" t="n"/>
       <c r="N58" s="6" t="n"/>
-      <c r="O58" s="7" t="n"/>
-      <c r="P58" s="6" t="n"/>
+      <c r="O58" s="6" t="n"/>
+      <c r="P58" s="7" t="n"/>
       <c r="Q58" s="6" t="n"/>
-      <c r="R58" s="7" t="n"/>
-      <c r="S58" s="3" t="inlineStr">
+      <c r="R58" s="6" t="n"/>
+      <c r="S58" s="7" t="n"/>
+      <c r="T58" s="3" t="inlineStr">
         <is>
           <t>387</t>
         </is>
       </c>
-      <c r="T58" s="3" t="inlineStr">
+      <c r="U58" s="3" t="inlineStr">
         <is>
           <t>388</t>
         </is>
@@ -4585,16 +4648,17 @@
       </c>
       <c r="M59" s="6" t="n"/>
       <c r="N59" s="6" t="n"/>
-      <c r="O59" s="7" t="n"/>
-      <c r="P59" s="6" t="n"/>
+      <c r="O59" s="6" t="n"/>
+      <c r="P59" s="7" t="n"/>
       <c r="Q59" s="6" t="n"/>
-      <c r="R59" s="7" t="n"/>
-      <c r="S59" s="3" t="inlineStr">
+      <c r="R59" s="6" t="n"/>
+      <c r="S59" s="7" t="n"/>
+      <c r="T59" s="3" t="inlineStr">
         <is>
           <t>922</t>
         </is>
       </c>
-      <c r="T59" s="3" t="inlineStr">
+      <c r="U59" s="3" t="inlineStr">
         <is>
           <t>924</t>
         </is>
@@ -4655,16 +4719,17 @@
       </c>
       <c r="M60" s="6" t="n"/>
       <c r="N60" s="6" t="n"/>
-      <c r="O60" s="7" t="n"/>
-      <c r="P60" s="6" t="n"/>
+      <c r="O60" s="6" t="n"/>
+      <c r="P60" s="7" t="n"/>
       <c r="Q60" s="6" t="n"/>
-      <c r="R60" s="7" t="n"/>
-      <c r="S60" s="3" t="inlineStr">
+      <c r="R60" s="6" t="n"/>
+      <c r="S60" s="7" t="n"/>
+      <c r="T60" s="3" t="inlineStr">
         <is>
           <t>845</t>
         </is>
       </c>
-      <c r="T60" s="3" t="inlineStr">
+      <c r="U60" s="3" t="inlineStr">
         <is>
           <t>847</t>
         </is>
@@ -4721,16 +4786,17 @@
       </c>
       <c r="M61" s="6" t="n"/>
       <c r="N61" s="6" t="n"/>
-      <c r="O61" s="7" t="n"/>
-      <c r="P61" s="6" t="n"/>
+      <c r="O61" s="6" t="n"/>
+      <c r="P61" s="7" t="n"/>
       <c r="Q61" s="6" t="n"/>
-      <c r="R61" s="7" t="n"/>
-      <c r="S61" s="3" t="inlineStr">
+      <c r="R61" s="6" t="n"/>
+      <c r="S61" s="7" t="n"/>
+      <c r="T61" s="3" t="inlineStr">
         <is>
           <t>263</t>
         </is>
       </c>
-      <c r="T61" s="3" t="inlineStr">
+      <c r="U61" s="3" t="inlineStr">
         <is>
           <t>264</t>
         </is>
@@ -4791,16 +4857,17 @@
       </c>
       <c r="M62" s="6" t="n"/>
       <c r="N62" s="6" t="n"/>
-      <c r="O62" s="7" t="n"/>
-      <c r="P62" s="6" t="n"/>
+      <c r="O62" s="6" t="n"/>
+      <c r="P62" s="7" t="n"/>
       <c r="Q62" s="6" t="n"/>
-      <c r="R62" s="7" t="n"/>
-      <c r="S62" s="3" t="inlineStr">
+      <c r="R62" s="6" t="n"/>
+      <c r="S62" s="7" t="n"/>
+      <c r="T62" s="3" t="inlineStr">
         <is>
           <t>237</t>
         </is>
       </c>
-      <c r="T62" s="3" t="inlineStr">
+      <c r="U62" s="3" t="inlineStr">
         <is>
           <t>238</t>
         </is>
@@ -4861,16 +4928,17 @@
       </c>
       <c r="M63" s="6" t="n"/>
       <c r="N63" s="6" t="n"/>
-      <c r="O63" s="7" t="n"/>
-      <c r="P63" s="6" t="n"/>
+      <c r="O63" s="6" t="n"/>
+      <c r="P63" s="7" t="n"/>
       <c r="Q63" s="6" t="n"/>
-      <c r="R63" s="7" t="n"/>
-      <c r="S63" s="3" t="inlineStr">
+      <c r="R63" s="6" t="n"/>
+      <c r="S63" s="7" t="n"/>
+      <c r="T63" s="3" t="inlineStr">
         <is>
           <t>213</t>
         </is>
       </c>
-      <c r="T63" s="3" t="inlineStr">
+      <c r="U63" s="3" t="inlineStr">
         <is>
           <t>214</t>
         </is>
@@ -4927,16 +4995,17 @@
       </c>
       <c r="M64" s="6" t="n"/>
       <c r="N64" s="6" t="n"/>
-      <c r="O64" s="7" t="n"/>
-      <c r="P64" s="6" t="n"/>
+      <c r="O64" s="6" t="n"/>
+      <c r="P64" s="7" t="n"/>
       <c r="Q64" s="6" t="n"/>
-      <c r="R64" s="7" t="n"/>
-      <c r="S64" s="3" t="inlineStr">
+      <c r="R64" s="6" t="n"/>
+      <c r="S64" s="7" t="n"/>
+      <c r="T64" s="3" t="inlineStr">
         <is>
           <t>453</t>
         </is>
       </c>
-      <c r="T64" s="3" t="inlineStr">
+      <c r="U64" s="3" t="inlineStr">
         <is>
           <t>454</t>
         </is>
@@ -4997,16 +5066,17 @@
       </c>
       <c r="M65" s="6" t="n"/>
       <c r="N65" s="6" t="n"/>
-      <c r="O65" s="7" t="n"/>
-      <c r="P65" s="6" t="n"/>
+      <c r="O65" s="6" t="n"/>
+      <c r="P65" s="7" t="n"/>
       <c r="Q65" s="6" t="n"/>
-      <c r="R65" s="7" t="n"/>
-      <c r="S65" s="3" t="inlineStr">
+      <c r="R65" s="6" t="n"/>
+      <c r="S65" s="7" t="n"/>
+      <c r="T65" s="3" t="inlineStr">
         <is>
           <t>898</t>
         </is>
       </c>
-      <c r="T65" s="3" t="inlineStr">
+      <c r="U65" s="3" t="inlineStr">
         <is>
           <t>900</t>
         </is>
@@ -5067,16 +5137,17 @@
       </c>
       <c r="M66" s="6" t="n"/>
       <c r="N66" s="6" t="n"/>
-      <c r="O66" s="7" t="n"/>
-      <c r="P66" s="6" t="n"/>
+      <c r="O66" s="6" t="n"/>
+      <c r="P66" s="7" t="n"/>
       <c r="Q66" s="6" t="n"/>
-      <c r="R66" s="7" t="n"/>
-      <c r="S66" s="3" t="inlineStr">
+      <c r="R66" s="6" t="n"/>
+      <c r="S66" s="7" t="n"/>
+      <c r="T66" s="3" t="inlineStr">
         <is>
           <t>802</t>
         </is>
       </c>
-      <c r="T66" s="3" t="inlineStr">
+      <c r="U66" s="3" t="inlineStr">
         <is>
           <t>803</t>
         </is>
@@ -5137,16 +5208,17 @@
       </c>
       <c r="M67" s="6" t="n"/>
       <c r="N67" s="6" t="n"/>
-      <c r="O67" s="7" t="n"/>
-      <c r="P67" s="6" t="n"/>
+      <c r="O67" s="6" t="n"/>
+      <c r="P67" s="7" t="n"/>
       <c r="Q67" s="6" t="n"/>
-      <c r="R67" s="7" t="n"/>
-      <c r="S67" s="3" t="inlineStr">
+      <c r="R67" s="6" t="n"/>
+      <c r="S67" s="7" t="n"/>
+      <c r="T67" s="3" t="inlineStr">
         <is>
           <t>614</t>
         </is>
       </c>
-      <c r="T67" s="3" t="inlineStr">
+      <c r="U67" s="3" t="inlineStr">
         <is>
           <t>615</t>
         </is>
@@ -5207,16 +5279,17 @@
       </c>
       <c r="M68" s="6" t="n"/>
       <c r="N68" s="6" t="n"/>
-      <c r="O68" s="7" t="n"/>
-      <c r="P68" s="6" t="n"/>
+      <c r="O68" s="6" t="n"/>
+      <c r="P68" s="7" t="n"/>
       <c r="Q68" s="6" t="n"/>
-      <c r="R68" s="7" t="n"/>
-      <c r="S68" s="3" t="inlineStr">
+      <c r="R68" s="6" t="n"/>
+      <c r="S68" s="7" t="n"/>
+      <c r="T68" s="3" t="inlineStr">
         <is>
           <t>796</t>
         </is>
       </c>
-      <c r="T68" s="3" t="inlineStr">
+      <c r="U68" s="3" t="inlineStr">
         <is>
           <t>797</t>
         </is>
@@ -5277,16 +5350,17 @@
       </c>
       <c r="M69" s="6" t="n"/>
       <c r="N69" s="6" t="n"/>
-      <c r="O69" s="7" t="n"/>
-      <c r="P69" s="6" t="n"/>
+      <c r="O69" s="6" t="n"/>
+      <c r="P69" s="7" t="n"/>
       <c r="Q69" s="6" t="n"/>
-      <c r="R69" s="7" t="n"/>
-      <c r="S69" s="3" t="inlineStr">
+      <c r="R69" s="6" t="n"/>
+      <c r="S69" s="7" t="n"/>
+      <c r="T69" s="3" t="inlineStr">
         <is>
           <t>959</t>
         </is>
       </c>
-      <c r="T69" s="3" t="inlineStr">
+      <c r="U69" s="3" t="inlineStr">
         <is>
           <t>961</t>
         </is>
@@ -5343,16 +5417,17 @@
       </c>
       <c r="M70" s="6" t="n"/>
       <c r="N70" s="6" t="n"/>
-      <c r="O70" s="7" t="n"/>
-      <c r="P70" s="6" t="n"/>
+      <c r="O70" s="6" t="n"/>
+      <c r="P70" s="7" t="n"/>
       <c r="Q70" s="6" t="n"/>
-      <c r="R70" s="7" t="n"/>
-      <c r="S70" s="3" t="inlineStr">
+      <c r="R70" s="6" t="n"/>
+      <c r="S70" s="7" t="n"/>
+      <c r="T70" s="3" t="inlineStr">
         <is>
           <t>449</t>
         </is>
       </c>
-      <c r="T70" s="3" t="inlineStr">
+      <c r="U70" s="3" t="inlineStr">
         <is>
           <t>450</t>
         </is>
@@ -5413,16 +5488,17 @@
       </c>
       <c r="M71" s="6" t="n"/>
       <c r="N71" s="6" t="n"/>
-      <c r="O71" s="7" t="n"/>
-      <c r="P71" s="6" t="n"/>
+      <c r="O71" s="6" t="n"/>
+      <c r="P71" s="7" t="n"/>
       <c r="Q71" s="6" t="n"/>
-      <c r="R71" s="7" t="n"/>
-      <c r="S71" s="3" t="inlineStr">
+      <c r="R71" s="6" t="n"/>
+      <c r="S71" s="7" t="n"/>
+      <c r="T71" s="3" t="inlineStr">
         <is>
           <t>820</t>
         </is>
       </c>
-      <c r="T71" s="3" t="inlineStr">
+      <c r="U71" s="3" t="inlineStr">
         <is>
           <t>822</t>
         </is>
@@ -5483,16 +5559,17 @@
       </c>
       <c r="M72" s="6" t="n"/>
       <c r="N72" s="6" t="n"/>
-      <c r="O72" s="7" t="n"/>
-      <c r="P72" s="6" t="n"/>
+      <c r="O72" s="6" t="n"/>
+      <c r="P72" s="7" t="n"/>
       <c r="Q72" s="6" t="n"/>
-      <c r="R72" s="7" t="n"/>
-      <c r="S72" s="3" t="inlineStr">
+      <c r="R72" s="6" t="n"/>
+      <c r="S72" s="7" t="n"/>
+      <c r="T72" s="3" t="inlineStr">
         <is>
           <t>783</t>
         </is>
       </c>
-      <c r="T72" s="3" t="inlineStr">
+      <c r="U72" s="3" t="inlineStr">
         <is>
           <t>784</t>
         </is>
@@ -5549,16 +5626,17 @@
       </c>
       <c r="M73" s="6" t="n"/>
       <c r="N73" s="6" t="n"/>
-      <c r="O73" s="7" t="n"/>
-      <c r="P73" s="6" t="n"/>
+      <c r="O73" s="6" t="n"/>
+      <c r="P73" s="7" t="n"/>
       <c r="Q73" s="6" t="n"/>
-      <c r="R73" s="7" t="n"/>
-      <c r="S73" s="3" t="inlineStr">
+      <c r="R73" s="6" t="n"/>
+      <c r="S73" s="7" t="n"/>
+      <c r="T73" s="3" t="inlineStr">
         <is>
           <t>442</t>
         </is>
       </c>
-      <c r="T73" s="3" t="inlineStr">
+      <c r="U73" s="3" t="inlineStr">
         <is>
           <t>443</t>
         </is>
@@ -5619,16 +5697,17 @@
       </c>
       <c r="M74" s="6" t="n"/>
       <c r="N74" s="6" t="n"/>
-      <c r="O74" s="7" t="n"/>
-      <c r="P74" s="6" t="n"/>
+      <c r="O74" s="6" t="n"/>
+      <c r="P74" s="7" t="n"/>
       <c r="Q74" s="6" t="n"/>
-      <c r="R74" s="7" t="n"/>
-      <c r="S74" s="3" t="inlineStr">
+      <c r="R74" s="6" t="n"/>
+      <c r="S74" s="7" t="n"/>
+      <c r="T74" s="3" t="inlineStr">
         <is>
           <t>513</t>
         </is>
       </c>
-      <c r="T74" s="3" t="inlineStr">
+      <c r="U74" s="3" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -5689,16 +5768,17 @@
       </c>
       <c r="M75" s="6" t="n"/>
       <c r="N75" s="6" t="n"/>
-      <c r="O75" s="7" t="n"/>
-      <c r="P75" s="6" t="n"/>
+      <c r="O75" s="6" t="n"/>
+      <c r="P75" s="7" t="n"/>
       <c r="Q75" s="6" t="n"/>
-      <c r="R75" s="7" t="n"/>
-      <c r="S75" s="3" t="inlineStr">
+      <c r="R75" s="6" t="n"/>
+      <c r="S75" s="7" t="n"/>
+      <c r="T75" s="3" t="inlineStr">
         <is>
           <t>311</t>
         </is>
       </c>
-      <c r="T75" s="3" t="inlineStr">
+      <c r="U75" s="3" t="inlineStr">
         <is>
           <t>312</t>
         </is>
@@ -5759,16 +5839,17 @@
       </c>
       <c r="M76" s="6" t="n"/>
       <c r="N76" s="6" t="n"/>
-      <c r="O76" s="7" t="n"/>
-      <c r="P76" s="6" t="n"/>
+      <c r="O76" s="6" t="n"/>
+      <c r="P76" s="7" t="n"/>
       <c r="Q76" s="6" t="n"/>
-      <c r="R76" s="7" t="n"/>
-      <c r="S76" s="3" t="inlineStr">
+      <c r="R76" s="6" t="n"/>
+      <c r="S76" s="7" t="n"/>
+      <c r="T76" s="3" t="inlineStr">
         <is>
           <t>980</t>
         </is>
       </c>
-      <c r="T76" s="3" t="inlineStr">
+      <c r="U76" s="3" t="inlineStr">
         <is>
           <t>982</t>
         </is>
@@ -5829,16 +5910,17 @@
       </c>
       <c r="M77" s="6" t="n"/>
       <c r="N77" s="6" t="n"/>
-      <c r="O77" s="7" t="n"/>
-      <c r="P77" s="6" t="n"/>
+      <c r="O77" s="6" t="n"/>
+      <c r="P77" s="7" t="n"/>
       <c r="Q77" s="6" t="n"/>
-      <c r="R77" s="7" t="n"/>
-      <c r="S77" s="3" t="inlineStr">
+      <c r="R77" s="6" t="n"/>
+      <c r="S77" s="7" t="n"/>
+      <c r="T77" s="3" t="inlineStr">
         <is>
           <t>662</t>
         </is>
       </c>
-      <c r="T77" s="3" t="inlineStr">
+      <c r="U77" s="3" t="inlineStr">
         <is>
           <t>663</t>
         </is>
@@ -5899,16 +5981,17 @@
       </c>
       <c r="M78" s="6" t="n"/>
       <c r="N78" s="6" t="n"/>
-      <c r="O78" s="7" t="n"/>
-      <c r="P78" s="6" t="n"/>
+      <c r="O78" s="6" t="n"/>
+      <c r="P78" s="7" t="n"/>
       <c r="Q78" s="6" t="n"/>
-      <c r="R78" s="7" t="n"/>
-      <c r="S78" s="3" t="inlineStr">
+      <c r="R78" s="6" t="n"/>
+      <c r="S78" s="7" t="n"/>
+      <c r="T78" s="3" t="inlineStr">
         <is>
           <t>837</t>
         </is>
       </c>
-      <c r="T78" s="3" t="inlineStr">
+      <c r="U78" s="3" t="inlineStr">
         <is>
           <t>839</t>
         </is>
@@ -5969,16 +6052,17 @@
       </c>
       <c r="M79" s="6" t="n"/>
       <c r="N79" s="6" t="n"/>
-      <c r="O79" s="7" t="n"/>
-      <c r="P79" s="6" t="n"/>
+      <c r="O79" s="6" t="n"/>
+      <c r="P79" s="7" t="n"/>
       <c r="Q79" s="6" t="n"/>
-      <c r="R79" s="7" t="n"/>
-      <c r="S79" s="3" t="inlineStr">
+      <c r="R79" s="6" t="n"/>
+      <c r="S79" s="7" t="n"/>
+      <c r="T79" s="3" t="inlineStr">
         <is>
           <t>391</t>
         </is>
       </c>
-      <c r="T79" s="3" t="inlineStr">
+      <c r="U79" s="3" t="inlineStr">
         <is>
           <t>392</t>
         </is>
@@ -6039,16 +6123,17 @@
       </c>
       <c r="M80" s="12" t="n"/>
       <c r="N80" s="12" t="n"/>
-      <c r="O80" s="13" t="n"/>
-      <c r="P80" s="12" t="n"/>
+      <c r="O80" s="12" t="n"/>
+      <c r="P80" s="13" t="n"/>
       <c r="Q80" s="12" t="n"/>
-      <c r="R80" s="13" t="n"/>
-      <c r="S80" s="9" t="inlineStr">
+      <c r="R80" s="12" t="n"/>
+      <c r="S80" s="13" t="n"/>
+      <c r="T80" s="9" t="inlineStr">
         <is>
           <t>441</t>
         </is>
       </c>
-      <c r="T80" s="9" t="inlineStr">
+      <c r="U80" s="9" t="inlineStr">
         <is>
           <t>442</t>
         </is>
@@ -6109,16 +6194,17 @@
       </c>
       <c r="M81" s="6" t="n"/>
       <c r="N81" s="6" t="n"/>
-      <c r="O81" s="7" t="n"/>
-      <c r="P81" s="6" t="n"/>
+      <c r="O81" s="6" t="n"/>
+      <c r="P81" s="7" t="n"/>
       <c r="Q81" s="6" t="n"/>
-      <c r="R81" s="7" t="n"/>
-      <c r="S81" s="3" t="inlineStr">
+      <c r="R81" s="6" t="n"/>
+      <c r="S81" s="7" t="n"/>
+      <c r="T81" s="3" t="inlineStr">
         <is>
           <t>68</t>
         </is>
       </c>
-      <c r="T81" s="3" t="inlineStr">
+      <c r="U81" s="3" t="inlineStr">
         <is>
           <t>68</t>
         </is>
@@ -6179,16 +6265,17 @@
       </c>
       <c r="M82" s="6" t="n"/>
       <c r="N82" s="6" t="n"/>
-      <c r="O82" s="7" t="n"/>
-      <c r="P82" s="6" t="n"/>
+      <c r="O82" s="6" t="n"/>
+      <c r="P82" s="7" t="n"/>
       <c r="Q82" s="6" t="n"/>
-      <c r="R82" s="7" t="n"/>
-      <c r="S82" s="3" t="inlineStr">
+      <c r="R82" s="6" t="n"/>
+      <c r="S82" s="7" t="n"/>
+      <c r="T82" s="3" t="inlineStr">
         <is>
           <t>547</t>
         </is>
       </c>
-      <c r="T82" s="3" t="inlineStr">
+      <c r="U82" s="3" t="inlineStr">
         <is>
           <t>548</t>
         </is>
@@ -6249,16 +6336,17 @@
       </c>
       <c r="M83" s="6" t="n"/>
       <c r="N83" s="6" t="n"/>
-      <c r="O83" s="7" t="n"/>
-      <c r="P83" s="6" t="n"/>
+      <c r="O83" s="6" t="n"/>
+      <c r="P83" s="7" t="n"/>
       <c r="Q83" s="6" t="n"/>
-      <c r="R83" s="7" t="n"/>
-      <c r="S83" s="3" t="inlineStr">
+      <c r="R83" s="6" t="n"/>
+      <c r="S83" s="7" t="n"/>
+      <c r="T83" s="3" t="inlineStr">
         <is>
           <t>428</t>
         </is>
       </c>
-      <c r="T83" s="3" t="inlineStr">
+      <c r="U83" s="3" t="inlineStr">
         <is>
           <t>429</t>
         </is>
@@ -6319,16 +6407,17 @@
       </c>
       <c r="M84" s="6" t="n"/>
       <c r="N84" s="6" t="n"/>
-      <c r="O84" s="7" t="n"/>
-      <c r="P84" s="6" t="n"/>
+      <c r="O84" s="6" t="n"/>
+      <c r="P84" s="7" t="n"/>
       <c r="Q84" s="6" t="n"/>
-      <c r="R84" s="7" t="n"/>
-      <c r="S84" s="3" t="inlineStr">
+      <c r="R84" s="6" t="n"/>
+      <c r="S84" s="7" t="n"/>
+      <c r="T84" s="3" t="inlineStr">
         <is>
           <t>979</t>
         </is>
       </c>
-      <c r="T84" s="3" t="inlineStr">
+      <c r="U84" s="3" t="inlineStr">
         <is>
           <t>981</t>
         </is>
@@ -6385,16 +6474,17 @@
       </c>
       <c r="M85" s="6" t="n"/>
       <c r="N85" s="6" t="n"/>
-      <c r="O85" s="7" t="n"/>
-      <c r="P85" s="6" t="n"/>
+      <c r="O85" s="6" t="n"/>
+      <c r="P85" s="7" t="n"/>
       <c r="Q85" s="6" t="n"/>
-      <c r="R85" s="7" t="n"/>
-      <c r="S85" s="3" t="inlineStr">
+      <c r="R85" s="6" t="n"/>
+      <c r="S85" s="7" t="n"/>
+      <c r="T85" s="3" t="inlineStr">
         <is>
           <t>731</t>
         </is>
       </c>
-      <c r="T85" s="3" t="inlineStr">
+      <c r="U85" s="3" t="inlineStr">
         <is>
           <t>732</t>
         </is>
@@ -6451,16 +6541,17 @@
       </c>
       <c r="M86" s="6" t="n"/>
       <c r="N86" s="6" t="n"/>
-      <c r="O86" s="7" t="n"/>
-      <c r="P86" s="6" t="n"/>
+      <c r="O86" s="6" t="n"/>
+      <c r="P86" s="7" t="n"/>
       <c r="Q86" s="6" t="n"/>
-      <c r="R86" s="7" t="n"/>
-      <c r="S86" s="3" t="inlineStr">
+      <c r="R86" s="6" t="n"/>
+      <c r="S86" s="7" t="n"/>
+      <c r="T86" s="3" t="inlineStr">
         <is>
           <t>1026</t>
         </is>
       </c>
-      <c r="T86" s="3" t="inlineStr">
+      <c r="U86" s="3" t="inlineStr">
         <is>
           <t>1028</t>
         </is>
@@ -6521,16 +6612,17 @@
       </c>
       <c r="M87" s="6" t="n"/>
       <c r="N87" s="6" t="n"/>
-      <c r="O87" s="7" t="n"/>
-      <c r="P87" s="6" t="n"/>
+      <c r="O87" s="6" t="n"/>
+      <c r="P87" s="7" t="n"/>
       <c r="Q87" s="6" t="n"/>
-      <c r="R87" s="7" t="n"/>
-      <c r="S87" s="3" t="inlineStr">
+      <c r="R87" s="6" t="n"/>
+      <c r="S87" s="7" t="n"/>
+      <c r="T87" s="3" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="T87" s="3" t="inlineStr">
+      <c r="U87" s="3" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -6591,16 +6683,17 @@
       </c>
       <c r="M88" s="6" t="n"/>
       <c r="N88" s="6" t="n"/>
-      <c r="O88" s="7" t="n"/>
-      <c r="P88" s="6" t="n"/>
+      <c r="O88" s="6" t="n"/>
+      <c r="P88" s="7" t="n"/>
       <c r="Q88" s="6" t="n"/>
-      <c r="R88" s="7" t="n"/>
-      <c r="S88" s="3" t="inlineStr">
+      <c r="R88" s="6" t="n"/>
+      <c r="S88" s="7" t="n"/>
+      <c r="T88" s="3" t="inlineStr">
         <is>
           <t>83</t>
         </is>
       </c>
-      <c r="T88" s="3" t="inlineStr">
+      <c r="U88" s="3" t="inlineStr">
         <is>
           <t>83</t>
         </is>
@@ -6661,16 +6754,17 @@
       </c>
       <c r="M89" s="6" t="n"/>
       <c r="N89" s="6" t="n"/>
-      <c r="O89" s="7" t="n"/>
-      <c r="P89" s="6" t="n"/>
+      <c r="O89" s="6" t="n"/>
+      <c r="P89" s="7" t="n"/>
       <c r="Q89" s="6" t="n"/>
-      <c r="R89" s="7" t="n"/>
-      <c r="S89" s="3" t="inlineStr">
+      <c r="R89" s="6" t="n"/>
+      <c r="S89" s="7" t="n"/>
+      <c r="T89" s="3" t="inlineStr">
         <is>
           <t>679</t>
         </is>
       </c>
-      <c r="T89" s="3" t="inlineStr">
+      <c r="U89" s="3" t="inlineStr">
         <is>
           <t>680</t>
         </is>
@@ -6731,16 +6825,17 @@
       </c>
       <c r="M90" s="6" t="n"/>
       <c r="N90" s="6" t="n"/>
-      <c r="O90" s="7" t="n"/>
-      <c r="P90" s="6" t="n"/>
+      <c r="O90" s="6" t="n"/>
+      <c r="P90" s="7" t="n"/>
       <c r="Q90" s="6" t="n"/>
-      <c r="R90" s="7" t="n"/>
-      <c r="S90" s="3" t="inlineStr">
+      <c r="R90" s="6" t="n"/>
+      <c r="S90" s="7" t="n"/>
+      <c r="T90" s="3" t="inlineStr">
         <is>
           <t>489</t>
         </is>
       </c>
-      <c r="T90" s="3" t="inlineStr">
+      <c r="U90" s="3" t="inlineStr">
         <is>
           <t>490</t>
         </is>
@@ -6789,7 +6884,11 @@
       <c r="J91" s="3" t="n">
         <v>0.3</v>
       </c>
-      <c r="K91" s="3" t="n"/>
+      <c r="K91" s="5" t="inlineStr">
+        <is>
+          <t>open profile</t>
+        </is>
+      </c>
       <c r="L91" s="5" t="inlineStr">
         <is>
           <t>open site</t>
@@ -6797,16 +6896,17 @@
       </c>
       <c r="M91" s="6" t="n"/>
       <c r="N91" s="6" t="n"/>
-      <c r="O91" s="7" t="n"/>
-      <c r="P91" s="6" t="n"/>
+      <c r="O91" s="6" t="n"/>
+      <c r="P91" s="7" t="n"/>
       <c r="Q91" s="6" t="n"/>
-      <c r="R91" s="7" t="n"/>
-      <c r="S91" s="3" t="inlineStr">
+      <c r="R91" s="6" t="n"/>
+      <c r="S91" s="7" t="n"/>
+      <c r="T91" s="3" t="inlineStr">
         <is>
           <t>730</t>
         </is>
       </c>
-      <c r="T91" s="3" t="inlineStr">
+      <c r="U91" s="3" t="inlineStr">
         <is>
           <t>731</t>
         </is>
@@ -6863,16 +6963,17 @@
       </c>
       <c r="M92" s="6" t="n"/>
       <c r="N92" s="6" t="n"/>
-      <c r="O92" s="7" t="n"/>
-      <c r="P92" s="6" t="n"/>
+      <c r="O92" s="6" t="n"/>
+      <c r="P92" s="7" t="n"/>
       <c r="Q92" s="6" t="n"/>
-      <c r="R92" s="7" t="n"/>
-      <c r="S92" s="3" t="inlineStr">
+      <c r="R92" s="6" t="n"/>
+      <c r="S92" s="7" t="n"/>
+      <c r="T92" s="3" t="inlineStr">
         <is>
           <t>704</t>
         </is>
       </c>
-      <c r="T92" s="3" t="inlineStr">
+      <c r="U92" s="3" t="inlineStr">
         <is>
           <t>705</t>
         </is>
@@ -6933,16 +7034,17 @@
       </c>
       <c r="M93" s="6" t="n"/>
       <c r="N93" s="6" t="n"/>
-      <c r="O93" s="7" t="n"/>
-      <c r="P93" s="6" t="n"/>
+      <c r="O93" s="6" t="n"/>
+      <c r="P93" s="7" t="n"/>
       <c r="Q93" s="6" t="n"/>
-      <c r="R93" s="7" t="n"/>
-      <c r="S93" s="3" t="inlineStr">
+      <c r="R93" s="6" t="n"/>
+      <c r="S93" s="7" t="n"/>
+      <c r="T93" s="3" t="inlineStr">
         <is>
           <t>602</t>
         </is>
       </c>
-      <c r="T93" s="3" t="inlineStr">
+      <c r="U93" s="3" t="inlineStr">
         <is>
           <t>603</t>
         </is>
@@ -7003,16 +7105,17 @@
       </c>
       <c r="M94" s="6" t="n"/>
       <c r="N94" s="6" t="n"/>
-      <c r="O94" s="7" t="n"/>
-      <c r="P94" s="6" t="n"/>
+      <c r="O94" s="6" t="n"/>
+      <c r="P94" s="7" t="n"/>
       <c r="Q94" s="6" t="n"/>
-      <c r="R94" s="7" t="n"/>
-      <c r="S94" s="3" t="inlineStr">
+      <c r="R94" s="6" t="n"/>
+      <c r="S94" s="7" t="n"/>
+      <c r="T94" s="3" t="inlineStr">
         <is>
           <t>273</t>
         </is>
       </c>
-      <c r="T94" s="3" t="inlineStr">
+      <c r="U94" s="3" t="inlineStr">
         <is>
           <t>274</t>
         </is>
@@ -7073,16 +7176,17 @@
       </c>
       <c r="M95" s="6" t="n"/>
       <c r="N95" s="6" t="n"/>
-      <c r="O95" s="7" t="n"/>
-      <c r="P95" s="6" t="n"/>
+      <c r="O95" s="6" t="n"/>
+      <c r="P95" s="7" t="n"/>
       <c r="Q95" s="6" t="n"/>
-      <c r="R95" s="7" t="n"/>
-      <c r="S95" s="3" t="inlineStr">
+      <c r="R95" s="6" t="n"/>
+      <c r="S95" s="7" t="n"/>
+      <c r="T95" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
       </c>
-      <c r="T95" s="3" t="inlineStr">
+      <c r="U95" s="3" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -7139,16 +7243,17 @@
       </c>
       <c r="M96" s="6" t="n"/>
       <c r="N96" s="6" t="n"/>
-      <c r="O96" s="7" t="n"/>
-      <c r="P96" s="6" t="n"/>
+      <c r="O96" s="6" t="n"/>
+      <c r="P96" s="7" t="n"/>
       <c r="Q96" s="6" t="n"/>
-      <c r="R96" s="7" t="n"/>
-      <c r="S96" s="3" t="inlineStr">
+      <c r="R96" s="6" t="n"/>
+      <c r="S96" s="7" t="n"/>
+      <c r="T96" s="3" t="inlineStr">
         <is>
           <t>913</t>
         </is>
       </c>
-      <c r="T96" s="3" t="inlineStr">
+      <c r="U96" s="3" t="inlineStr">
         <is>
           <t>915</t>
         </is>
@@ -7209,16 +7314,17 @@
       </c>
       <c r="M97" s="6" t="n"/>
       <c r="N97" s="6" t="n"/>
-      <c r="O97" s="7" t="n"/>
-      <c r="P97" s="6" t="n"/>
+      <c r="O97" s="6" t="n"/>
+      <c r="P97" s="7" t="n"/>
       <c r="Q97" s="6" t="n"/>
-      <c r="R97" s="7" t="n"/>
-      <c r="S97" s="3" t="inlineStr">
+      <c r="R97" s="6" t="n"/>
+      <c r="S97" s="7" t="n"/>
+      <c r="T97" s="3" t="inlineStr">
         <is>
           <t>912</t>
         </is>
       </c>
-      <c r="T97" s="3" t="inlineStr">
+      <c r="U97" s="3" t="inlineStr">
         <is>
           <t>914</t>
         </is>
@@ -7279,16 +7385,17 @@
       </c>
       <c r="M98" s="6" t="n"/>
       <c r="N98" s="6" t="n"/>
-      <c r="O98" s="7" t="n"/>
-      <c r="P98" s="6" t="n"/>
+      <c r="O98" s="6" t="n"/>
+      <c r="P98" s="7" t="n"/>
       <c r="Q98" s="6" t="n"/>
-      <c r="R98" s="7" t="n"/>
-      <c r="S98" s="3" t="inlineStr">
+      <c r="R98" s="6" t="n"/>
+      <c r="S98" s="7" t="n"/>
+      <c r="T98" s="3" t="inlineStr">
         <is>
           <t>754</t>
         </is>
       </c>
-      <c r="T98" s="3" t="inlineStr">
+      <c r="U98" s="3" t="inlineStr">
         <is>
           <t>755</t>
         </is>
@@ -7349,16 +7456,17 @@
       </c>
       <c r="M99" s="6" t="n"/>
       <c r="N99" s="6" t="n"/>
-      <c r="O99" s="7" t="n"/>
-      <c r="P99" s="6" t="n"/>
+      <c r="O99" s="6" t="n"/>
+      <c r="P99" s="7" t="n"/>
       <c r="Q99" s="6" t="n"/>
-      <c r="R99" s="7" t="n"/>
-      <c r="S99" s="3" t="inlineStr">
+      <c r="R99" s="6" t="n"/>
+      <c r="S99" s="7" t="n"/>
+      <c r="T99" s="3" t="inlineStr">
         <is>
           <t>923</t>
         </is>
       </c>
-      <c r="T99" s="3" t="inlineStr">
+      <c r="U99" s="3" t="inlineStr">
         <is>
           <t>925</t>
         </is>
@@ -7415,16 +7523,17 @@
       </c>
       <c r="M100" s="6" t="n"/>
       <c r="N100" s="6" t="n"/>
-      <c r="O100" s="7" t="n"/>
-      <c r="P100" s="6" t="n"/>
+      <c r="O100" s="6" t="n"/>
+      <c r="P100" s="7" t="n"/>
       <c r="Q100" s="6" t="n"/>
-      <c r="R100" s="7" t="n"/>
-      <c r="S100" s="3" t="inlineStr">
+      <c r="R100" s="6" t="n"/>
+      <c r="S100" s="7" t="n"/>
+      <c r="T100" s="3" t="inlineStr">
         <is>
           <t>480</t>
         </is>
       </c>
-      <c r="T100" s="3" t="inlineStr">
+      <c r="U100" s="3" t="inlineStr">
         <is>
           <t>481</t>
         </is>
@@ -7485,16 +7594,17 @@
       </c>
       <c r="M101" s="6" t="n"/>
       <c r="N101" s="6" t="n"/>
-      <c r="O101" s="7" t="n"/>
-      <c r="P101" s="6" t="n"/>
+      <c r="O101" s="6" t="n"/>
+      <c r="P101" s="7" t="n"/>
       <c r="Q101" s="6" t="n"/>
-      <c r="R101" s="7" t="n"/>
-      <c r="S101" s="3" t="inlineStr">
+      <c r="R101" s="6" t="n"/>
+      <c r="S101" s="7" t="n"/>
+      <c r="T101" s="3" t="inlineStr">
         <is>
           <t>733</t>
         </is>
       </c>
-      <c r="T101" s="3" t="inlineStr">
+      <c r="U101" s="3" t="inlineStr">
         <is>
           <t>734</t>
         </is>
@@ -7555,16 +7665,17 @@
       </c>
       <c r="M102" s="6" t="n"/>
       <c r="N102" s="6" t="n"/>
-      <c r="O102" s="7" t="n"/>
-      <c r="P102" s="6" t="n"/>
+      <c r="O102" s="6" t="n"/>
+      <c r="P102" s="7" t="n"/>
       <c r="Q102" s="6" t="n"/>
-      <c r="R102" s="7" t="n"/>
-      <c r="S102" s="3" t="inlineStr">
+      <c r="R102" s="6" t="n"/>
+      <c r="S102" s="7" t="n"/>
+      <c r="T102" s="3" t="inlineStr">
         <is>
           <t>581</t>
         </is>
       </c>
-      <c r="T102" s="3" t="inlineStr">
+      <c r="U102" s="3" t="inlineStr">
         <is>
           <t>582</t>
         </is>
@@ -7625,16 +7736,17 @@
       </c>
       <c r="M103" s="6" t="n"/>
       <c r="N103" s="6" t="n"/>
-      <c r="O103" s="7" t="n"/>
-      <c r="P103" s="6" t="n"/>
+      <c r="O103" s="6" t="n"/>
+      <c r="P103" s="7" t="n"/>
       <c r="Q103" s="6" t="n"/>
-      <c r="R103" s="7" t="n"/>
-      <c r="S103" s="3" t="inlineStr">
+      <c r="R103" s="6" t="n"/>
+      <c r="S103" s="7" t="n"/>
+      <c r="T103" s="3" t="inlineStr">
         <is>
           <t>77</t>
         </is>
       </c>
-      <c r="T103" s="3" t="inlineStr">
+      <c r="U103" s="3" t="inlineStr">
         <is>
           <t>77</t>
         </is>
@@ -7695,16 +7807,17 @@
       </c>
       <c r="M104" s="6" t="n"/>
       <c r="N104" s="6" t="n"/>
-      <c r="O104" s="7" t="n"/>
-      <c r="P104" s="6" t="n"/>
+      <c r="O104" s="6" t="n"/>
+      <c r="P104" s="7" t="n"/>
       <c r="Q104" s="6" t="n"/>
-      <c r="R104" s="7" t="n"/>
-      <c r="S104" s="3" t="inlineStr">
+      <c r="R104" s="6" t="n"/>
+      <c r="S104" s="7" t="n"/>
+      <c r="T104" s="3" t="inlineStr">
         <is>
           <t>778</t>
         </is>
       </c>
-      <c r="T104" s="3" t="inlineStr">
+      <c r="U104" s="3" t="inlineStr">
         <is>
           <t>779</t>
         </is>
@@ -7765,16 +7878,17 @@
       </c>
       <c r="M105" s="6" t="n"/>
       <c r="N105" s="6" t="n"/>
-      <c r="O105" s="7" t="n"/>
-      <c r="P105" s="6" t="n"/>
+      <c r="O105" s="6" t="n"/>
+      <c r="P105" s="7" t="n"/>
       <c r="Q105" s="6" t="n"/>
-      <c r="R105" s="7" t="n"/>
-      <c r="S105" s="3" t="inlineStr">
+      <c r="R105" s="6" t="n"/>
+      <c r="S105" s="7" t="n"/>
+      <c r="T105" s="3" t="inlineStr">
         <is>
           <t>162</t>
         </is>
       </c>
-      <c r="T105" s="3" t="inlineStr">
+      <c r="U105" s="3" t="inlineStr">
         <is>
           <t>163</t>
         </is>
@@ -7835,16 +7949,17 @@
       </c>
       <c r="M106" s="6" t="n"/>
       <c r="N106" s="6" t="n"/>
-      <c r="O106" s="7" t="n"/>
-      <c r="P106" s="6" t="n"/>
+      <c r="O106" s="6" t="n"/>
+      <c r="P106" s="7" t="n"/>
       <c r="Q106" s="6" t="n"/>
-      <c r="R106" s="7" t="n"/>
-      <c r="S106" s="3" t="inlineStr">
+      <c r="R106" s="6" t="n"/>
+      <c r="S106" s="7" t="n"/>
+      <c r="T106" s="3" t="inlineStr">
         <is>
           <t>701</t>
         </is>
       </c>
-      <c r="T106" s="3" t="inlineStr">
+      <c r="U106" s="3" t="inlineStr">
         <is>
           <t>702</t>
         </is>
@@ -7901,16 +8016,17 @@
       </c>
       <c r="M107" s="6" t="n"/>
       <c r="N107" s="6" t="n"/>
-      <c r="O107" s="7" t="n"/>
-      <c r="P107" s="6" t="n"/>
+      <c r="O107" s="6" t="n"/>
+      <c r="P107" s="7" t="n"/>
       <c r="Q107" s="6" t="n"/>
-      <c r="R107" s="7" t="n"/>
-      <c r="S107" s="3" t="inlineStr">
+      <c r="R107" s="6" t="n"/>
+      <c r="S107" s="7" t="n"/>
+      <c r="T107" s="3" t="inlineStr">
         <is>
           <t>466</t>
         </is>
       </c>
-      <c r="T107" s="3" t="inlineStr">
+      <c r="U107" s="3" t="inlineStr">
         <is>
           <t>467</t>
         </is>
@@ -7971,16 +8087,17 @@
       </c>
       <c r="M108" s="6" t="n"/>
       <c r="N108" s="6" t="n"/>
-      <c r="O108" s="7" t="n"/>
-      <c r="P108" s="6" t="n"/>
+      <c r="O108" s="6" t="n"/>
+      <c r="P108" s="7" t="n"/>
       <c r="Q108" s="6" t="n"/>
-      <c r="R108" s="7" t="n"/>
-      <c r="S108" s="3" t="inlineStr">
+      <c r="R108" s="6" t="n"/>
+      <c r="S108" s="7" t="n"/>
+      <c r="T108" s="3" t="inlineStr">
         <is>
           <t>958</t>
         </is>
       </c>
-      <c r="T108" s="3" t="inlineStr">
+      <c r="U108" s="3" t="inlineStr">
         <is>
           <t>960</t>
         </is>
@@ -8041,16 +8158,17 @@
       </c>
       <c r="M109" s="6" t="n"/>
       <c r="N109" s="6" t="n"/>
-      <c r="O109" s="7" t="n"/>
-      <c r="P109" s="6" t="n"/>
+      <c r="O109" s="6" t="n"/>
+      <c r="P109" s="7" t="n"/>
       <c r="Q109" s="6" t="n"/>
-      <c r="R109" s="7" t="n"/>
-      <c r="S109" s="3" t="inlineStr">
+      <c r="R109" s="6" t="n"/>
+      <c r="S109" s="7" t="n"/>
+      <c r="T109" s="3" t="inlineStr">
         <is>
           <t>150</t>
         </is>
       </c>
-      <c r="T109" s="3" t="inlineStr">
+      <c r="U109" s="3" t="inlineStr">
         <is>
           <t>151</t>
         </is>
@@ -8111,16 +8229,17 @@
       </c>
       <c r="M110" s="6" t="n"/>
       <c r="N110" s="6" t="n"/>
-      <c r="O110" s="7" t="n"/>
-      <c r="P110" s="6" t="n"/>
+      <c r="O110" s="6" t="n"/>
+      <c r="P110" s="7" t="n"/>
       <c r="Q110" s="6" t="n"/>
-      <c r="R110" s="7" t="n"/>
-      <c r="S110" s="3" t="inlineStr">
+      <c r="R110" s="6" t="n"/>
+      <c r="S110" s="7" t="n"/>
+      <c r="T110" s="3" t="inlineStr">
         <is>
           <t>488</t>
         </is>
       </c>
-      <c r="T110" s="3" t="inlineStr">
+      <c r="U110" s="3" t="inlineStr">
         <is>
           <t>489</t>
         </is>
@@ -8181,16 +8300,17 @@
       </c>
       <c r="M111" s="6" t="n"/>
       <c r="N111" s="6" t="n"/>
-      <c r="O111" s="7" t="n"/>
-      <c r="P111" s="6" t="n"/>
+      <c r="O111" s="6" t="n"/>
+      <c r="P111" s="7" t="n"/>
       <c r="Q111" s="6" t="n"/>
-      <c r="R111" s="7" t="n"/>
-      <c r="S111" s="3" t="inlineStr">
+      <c r="R111" s="6" t="n"/>
+      <c r="S111" s="7" t="n"/>
+      <c r="T111" s="3" t="inlineStr">
         <is>
           <t>894</t>
         </is>
       </c>
-      <c r="T111" s="3" t="inlineStr">
+      <c r="U111" s="3" t="inlineStr">
         <is>
           <t>896</t>
         </is>
@@ -8251,16 +8371,17 @@
       </c>
       <c r="M112" s="6" t="n"/>
       <c r="N112" s="6" t="n"/>
-      <c r="O112" s="7" t="n"/>
-      <c r="P112" s="6" t="n"/>
+      <c r="O112" s="6" t="n"/>
+      <c r="P112" s="7" t="n"/>
       <c r="Q112" s="6" t="n"/>
-      <c r="R112" s="7" t="n"/>
-      <c r="S112" s="3" t="inlineStr">
+      <c r="R112" s="6" t="n"/>
+      <c r="S112" s="7" t="n"/>
+      <c r="T112" s="3" t="inlineStr">
         <is>
           <t>409</t>
         </is>
       </c>
-      <c r="T112" s="3" t="inlineStr">
+      <c r="U112" s="3" t="inlineStr">
         <is>
           <t>410</t>
         </is>
@@ -8321,16 +8442,17 @@
       </c>
       <c r="M113" s="6" t="n"/>
       <c r="N113" s="6" t="n"/>
-      <c r="O113" s="7" t="n"/>
-      <c r="P113" s="6" t="n"/>
+      <c r="O113" s="6" t="n"/>
+      <c r="P113" s="7" t="n"/>
       <c r="Q113" s="6" t="n"/>
-      <c r="R113" s="7" t="n"/>
-      <c r="S113" s="3" t="inlineStr">
+      <c r="R113" s="6" t="n"/>
+      <c r="S113" s="7" t="n"/>
+      <c r="T113" s="3" t="inlineStr">
         <is>
           <t>278</t>
         </is>
       </c>
-      <c r="T113" s="3" t="inlineStr">
+      <c r="U113" s="3" t="inlineStr">
         <is>
           <t>279</t>
         </is>
@@ -8387,16 +8509,17 @@
       </c>
       <c r="M114" s="6" t="n"/>
       <c r="N114" s="6" t="n"/>
-      <c r="O114" s="7" t="n"/>
-      <c r="P114" s="6" t="n"/>
+      <c r="O114" s="6" t="n"/>
+      <c r="P114" s="7" t="n"/>
       <c r="Q114" s="6" t="n"/>
-      <c r="R114" s="7" t="n"/>
-      <c r="S114" s="3" t="inlineStr">
+      <c r="R114" s="6" t="n"/>
+      <c r="S114" s="7" t="n"/>
+      <c r="T114" s="3" t="inlineStr">
         <is>
           <t>652</t>
         </is>
       </c>
-      <c r="T114" s="3" t="inlineStr">
+      <c r="U114" s="3" t="inlineStr">
         <is>
           <t>653</t>
         </is>
@@ -8457,16 +8580,17 @@
       </c>
       <c r="M115" s="6" t="n"/>
       <c r="N115" s="6" t="n"/>
-      <c r="O115" s="7" t="n"/>
-      <c r="P115" s="6" t="n"/>
+      <c r="O115" s="6" t="n"/>
+      <c r="P115" s="7" t="n"/>
       <c r="Q115" s="6" t="n"/>
-      <c r="R115" s="7" t="n"/>
-      <c r="S115" s="3" t="inlineStr">
+      <c r="R115" s="6" t="n"/>
+      <c r="S115" s="7" t="n"/>
+      <c r="T115" s="3" t="inlineStr">
         <is>
           <t>381</t>
         </is>
       </c>
-      <c r="T115" s="3" t="inlineStr">
+      <c r="U115" s="3" t="inlineStr">
         <is>
           <t>382</t>
         </is>
@@ -8527,16 +8651,17 @@
       </c>
       <c r="M116" s="6" t="n"/>
       <c r="N116" s="6" t="n"/>
-      <c r="O116" s="7" t="n"/>
-      <c r="P116" s="6" t="n"/>
+      <c r="O116" s="6" t="n"/>
+      <c r="P116" s="7" t="n"/>
       <c r="Q116" s="6" t="n"/>
-      <c r="R116" s="7" t="n"/>
-      <c r="S116" s="3" t="inlineStr">
+      <c r="R116" s="6" t="n"/>
+      <c r="S116" s="7" t="n"/>
+      <c r="T116" s="3" t="inlineStr">
         <is>
           <t>378</t>
         </is>
       </c>
-      <c r="T116" s="3" t="inlineStr">
+      <c r="U116" s="3" t="inlineStr">
         <is>
           <t>379</t>
         </is>
@@ -8593,16 +8718,17 @@
       </c>
       <c r="M117" s="6" t="n"/>
       <c r="N117" s="6" t="n"/>
-      <c r="O117" s="7" t="n"/>
-      <c r="P117" s="6" t="n"/>
+      <c r="O117" s="6" t="n"/>
+      <c r="P117" s="7" t="n"/>
       <c r="Q117" s="6" t="n"/>
-      <c r="R117" s="7" t="n"/>
-      <c r="S117" s="3" t="inlineStr">
+      <c r="R117" s="6" t="n"/>
+      <c r="S117" s="7" t="n"/>
+      <c r="T117" s="3" t="inlineStr">
         <is>
           <t>406</t>
         </is>
       </c>
-      <c r="T117" s="3" t="inlineStr">
+      <c r="U117" s="3" t="inlineStr">
         <is>
           <t>407</t>
         </is>
@@ -8663,16 +8789,17 @@
       </c>
       <c r="M118" s="6" t="n"/>
       <c r="N118" s="6" t="n"/>
-      <c r="O118" s="7" t="n"/>
-      <c r="P118" s="6" t="n"/>
+      <c r="O118" s="6" t="n"/>
+      <c r="P118" s="7" t="n"/>
       <c r="Q118" s="6" t="n"/>
-      <c r="R118" s="7" t="n"/>
-      <c r="S118" s="3" t="inlineStr">
+      <c r="R118" s="6" t="n"/>
+      <c r="S118" s="7" t="n"/>
+      <c r="T118" s="3" t="inlineStr">
         <is>
           <t>443</t>
         </is>
       </c>
-      <c r="T118" s="3" t="inlineStr">
+      <c r="U118" s="3" t="inlineStr">
         <is>
           <t>444</t>
         </is>
@@ -8733,16 +8860,17 @@
       </c>
       <c r="M119" s="6" t="n"/>
       <c r="N119" s="6" t="n"/>
-      <c r="O119" s="7" t="n"/>
-      <c r="P119" s="6" t="n"/>
+      <c r="O119" s="6" t="n"/>
+      <c r="P119" s="7" t="n"/>
       <c r="Q119" s="6" t="n"/>
-      <c r="R119" s="7" t="n"/>
-      <c r="S119" s="3" t="inlineStr">
+      <c r="R119" s="6" t="n"/>
+      <c r="S119" s="7" t="n"/>
+      <c r="T119" s="3" t="inlineStr">
         <is>
           <t>463</t>
         </is>
       </c>
-      <c r="T119" s="3" t="inlineStr">
+      <c r="U119" s="3" t="inlineStr">
         <is>
           <t>464</t>
         </is>
@@ -8803,16 +8931,17 @@
       </c>
       <c r="M120" s="6" t="n"/>
       <c r="N120" s="6" t="n"/>
-      <c r="O120" s="7" t="n"/>
-      <c r="P120" s="6" t="n"/>
+      <c r="O120" s="6" t="n"/>
+      <c r="P120" s="7" t="n"/>
       <c r="Q120" s="6" t="n"/>
-      <c r="R120" s="7" t="n"/>
-      <c r="S120" s="3" t="inlineStr">
+      <c r="R120" s="6" t="n"/>
+      <c r="S120" s="7" t="n"/>
+      <c r="T120" s="3" t="inlineStr">
         <is>
           <t>332</t>
         </is>
       </c>
-      <c r="T120" s="3" t="inlineStr">
+      <c r="U120" s="3" t="inlineStr">
         <is>
           <t>333</t>
         </is>
@@ -8873,16 +9002,17 @@
       </c>
       <c r="M121" s="6" t="n"/>
       <c r="N121" s="6" t="n"/>
-      <c r="O121" s="7" t="n"/>
-      <c r="P121" s="6" t="n"/>
+      <c r="O121" s="6" t="n"/>
+      <c r="P121" s="7" t="n"/>
       <c r="Q121" s="6" t="n"/>
-      <c r="R121" s="7" t="n"/>
-      <c r="S121" s="3" t="inlineStr">
+      <c r="R121" s="6" t="n"/>
+      <c r="S121" s="7" t="n"/>
+      <c r="T121" s="3" t="inlineStr">
         <is>
           <t>1017</t>
         </is>
       </c>
-      <c r="T121" s="3" t="inlineStr">
+      <c r="U121" s="3" t="inlineStr">
         <is>
           <t>1019</t>
         </is>
@@ -8939,16 +9069,17 @@
       </c>
       <c r="M122" s="6" t="n"/>
       <c r="N122" s="6" t="n"/>
-      <c r="O122" s="7" t="n"/>
-      <c r="P122" s="6" t="n"/>
+      <c r="O122" s="6" t="n"/>
+      <c r="P122" s="7" t="n"/>
       <c r="Q122" s="6" t="n"/>
-      <c r="R122" s="7" t="n"/>
-      <c r="S122" s="3" t="inlineStr">
+      <c r="R122" s="6" t="n"/>
+      <c r="S122" s="7" t="n"/>
+      <c r="T122" s="3" t="inlineStr">
         <is>
           <t>882</t>
         </is>
       </c>
-      <c r="T122" s="3" t="inlineStr">
+      <c r="U122" s="3" t="inlineStr">
         <is>
           <t>884</t>
         </is>
@@ -9005,16 +9136,17 @@
       </c>
       <c r="M123" s="6" t="n"/>
       <c r="N123" s="6" t="n"/>
-      <c r="O123" s="7" t="n"/>
-      <c r="P123" s="6" t="n"/>
+      <c r="O123" s="6" t="n"/>
+      <c r="P123" s="7" t="n"/>
       <c r="Q123" s="6" t="n"/>
-      <c r="R123" s="7" t="n"/>
-      <c r="S123" s="3" t="inlineStr">
+      <c r="R123" s="6" t="n"/>
+      <c r="S123" s="7" t="n"/>
+      <c r="T123" s="3" t="inlineStr">
         <is>
           <t>468</t>
         </is>
       </c>
-      <c r="T123" s="3" t="inlineStr">
+      <c r="U123" s="3" t="inlineStr">
         <is>
           <t>469</t>
         </is>
@@ -9075,16 +9207,17 @@
       </c>
       <c r="M124" s="6" t="n"/>
       <c r="N124" s="6" t="n"/>
-      <c r="O124" s="7" t="n"/>
-      <c r="P124" s="6" t="n"/>
+      <c r="O124" s="6" t="n"/>
+      <c r="P124" s="7" t="n"/>
       <c r="Q124" s="6" t="n"/>
-      <c r="R124" s="7" t="n"/>
-      <c r="S124" s="3" t="inlineStr">
+      <c r="R124" s="6" t="n"/>
+      <c r="S124" s="7" t="n"/>
+      <c r="T124" s="3" t="inlineStr">
         <is>
           <t>418</t>
         </is>
       </c>
-      <c r="T124" s="3" t="inlineStr">
+      <c r="U124" s="3" t="inlineStr">
         <is>
           <t>419</t>
         </is>
@@ -9141,16 +9274,17 @@
       </c>
       <c r="M125" s="6" t="n"/>
       <c r="N125" s="6" t="n"/>
-      <c r="O125" s="7" t="n"/>
-      <c r="P125" s="6" t="n"/>
+      <c r="O125" s="6" t="n"/>
+      <c r="P125" s="7" t="n"/>
       <c r="Q125" s="6" t="n"/>
-      <c r="R125" s="7" t="n"/>
-      <c r="S125" s="3" t="inlineStr">
+      <c r="R125" s="6" t="n"/>
+      <c r="S125" s="7" t="n"/>
+      <c r="T125" s="3" t="inlineStr">
         <is>
           <t>634</t>
         </is>
       </c>
-      <c r="T125" s="3" t="inlineStr">
+      <c r="U125" s="3" t="inlineStr">
         <is>
           <t>635</t>
         </is>
@@ -9207,16 +9341,17 @@
       </c>
       <c r="M126" s="6" t="n"/>
       <c r="N126" s="6" t="n"/>
-      <c r="O126" s="7" t="n"/>
-      <c r="P126" s="6" t="n"/>
+      <c r="O126" s="6" t="n"/>
+      <c r="P126" s="7" t="n"/>
       <c r="Q126" s="6" t="n"/>
-      <c r="R126" s="7" t="n"/>
-      <c r="S126" s="3" t="inlineStr">
+      <c r="R126" s="6" t="n"/>
+      <c r="S126" s="7" t="n"/>
+      <c r="T126" s="3" t="inlineStr">
         <is>
           <t>467</t>
         </is>
       </c>
-      <c r="T126" s="3" t="inlineStr">
+      <c r="U126" s="3" t="inlineStr">
         <is>
           <t>468</t>
         </is>
@@ -9277,16 +9412,17 @@
       </c>
       <c r="M127" s="6" t="n"/>
       <c r="N127" s="6" t="n"/>
-      <c r="O127" s="7" t="n"/>
-      <c r="P127" s="6" t="n"/>
+      <c r="O127" s="6" t="n"/>
+      <c r="P127" s="7" t="n"/>
       <c r="Q127" s="6" t="n"/>
-      <c r="R127" s="7" t="n"/>
-      <c r="S127" s="3" t="inlineStr">
+      <c r="R127" s="6" t="n"/>
+      <c r="S127" s="7" t="n"/>
+      <c r="T127" s="3" t="inlineStr">
         <is>
           <t>571</t>
         </is>
       </c>
-      <c r="T127" s="3" t="inlineStr">
+      <c r="U127" s="3" t="inlineStr">
         <is>
           <t>572</t>
         </is>
@@ -9347,16 +9483,17 @@
       </c>
       <c r="M128" s="6" t="n"/>
       <c r="N128" s="6" t="n"/>
-      <c r="O128" s="7" t="n"/>
-      <c r="P128" s="6" t="n"/>
+      <c r="O128" s="6" t="n"/>
+      <c r="P128" s="7" t="n"/>
       <c r="Q128" s="6" t="n"/>
-      <c r="R128" s="7" t="n"/>
-      <c r="S128" s="3" t="inlineStr">
+      <c r="R128" s="6" t="n"/>
+      <c r="S128" s="7" t="n"/>
+      <c r="T128" s="3" t="inlineStr">
         <is>
           <t>143</t>
         </is>
       </c>
-      <c r="T128" s="3" t="inlineStr">
+      <c r="U128" s="3" t="inlineStr">
         <is>
           <t>144</t>
         </is>
@@ -9413,16 +9550,17 @@
       </c>
       <c r="M129" s="6" t="n"/>
       <c r="N129" s="6" t="n"/>
-      <c r="O129" s="7" t="n"/>
-      <c r="P129" s="6" t="n"/>
+      <c r="O129" s="6" t="n"/>
+      <c r="P129" s="7" t="n"/>
       <c r="Q129" s="6" t="n"/>
-      <c r="R129" s="7" t="n"/>
-      <c r="S129" s="3" t="inlineStr">
+      <c r="R129" s="6" t="n"/>
+      <c r="S129" s="7" t="n"/>
+      <c r="T129" s="3" t="inlineStr">
         <is>
           <t>425</t>
         </is>
       </c>
-      <c r="T129" s="3" t="inlineStr">
+      <c r="U129" s="3" t="inlineStr">
         <is>
           <t>426</t>
         </is>
@@ -9483,16 +9621,17 @@
       </c>
       <c r="M130" s="6" t="n"/>
       <c r="N130" s="6" t="n"/>
-      <c r="O130" s="7" t="n"/>
-      <c r="P130" s="6" t="n"/>
+      <c r="O130" s="6" t="n"/>
+      <c r="P130" s="7" t="n"/>
       <c r="Q130" s="6" t="n"/>
-      <c r="R130" s="7" t="n"/>
-      <c r="S130" s="3" t="inlineStr">
+      <c r="R130" s="6" t="n"/>
+      <c r="S130" s="7" t="n"/>
+      <c r="T130" s="3" t="inlineStr">
         <is>
           <t>618</t>
         </is>
       </c>
-      <c r="T130" s="3" t="inlineStr">
+      <c r="U130" s="3" t="inlineStr">
         <is>
           <t>619</t>
         </is>
@@ -9553,16 +9692,17 @@
       </c>
       <c r="M131" s="6" t="n"/>
       <c r="N131" s="6" t="n"/>
-      <c r="O131" s="7" t="n"/>
-      <c r="P131" s="6" t="n"/>
+      <c r="O131" s="6" t="n"/>
+      <c r="P131" s="7" t="n"/>
       <c r="Q131" s="6" t="n"/>
-      <c r="R131" s="7" t="n"/>
-      <c r="S131" s="3" t="inlineStr">
+      <c r="R131" s="6" t="n"/>
+      <c r="S131" s="7" t="n"/>
+      <c r="T131" s="3" t="inlineStr">
         <is>
           <t>834</t>
         </is>
       </c>
-      <c r="T131" s="3" t="inlineStr">
+      <c r="U131" s="3" t="inlineStr">
         <is>
           <t>836</t>
         </is>
@@ -9623,16 +9763,17 @@
       </c>
       <c r="M132" s="6" t="n"/>
       <c r="N132" s="6" t="n"/>
-      <c r="O132" s="7" t="n"/>
-      <c r="P132" s="6" t="n"/>
+      <c r="O132" s="6" t="n"/>
+      <c r="P132" s="7" t="n"/>
       <c r="Q132" s="6" t="n"/>
-      <c r="R132" s="7" t="n"/>
-      <c r="S132" s="3" t="inlineStr">
+      <c r="R132" s="6" t="n"/>
+      <c r="S132" s="7" t="n"/>
+      <c r="T132" s="3" t="inlineStr">
         <is>
           <t>550</t>
         </is>
       </c>
-      <c r="T132" s="3" t="inlineStr">
+      <c r="U132" s="3" t="inlineStr">
         <is>
           <t>551</t>
         </is>
@@ -9693,16 +9834,17 @@
       </c>
       <c r="M133" s="6" t="n"/>
       <c r="N133" s="6" t="n"/>
-      <c r="O133" s="7" t="n"/>
-      <c r="P133" s="6" t="n"/>
+      <c r="O133" s="6" t="n"/>
+      <c r="P133" s="7" t="n"/>
       <c r="Q133" s="6" t="n"/>
-      <c r="R133" s="7" t="n"/>
-      <c r="S133" s="3" t="inlineStr">
+      <c r="R133" s="6" t="n"/>
+      <c r="S133" s="7" t="n"/>
+      <c r="T133" s="3" t="inlineStr">
         <is>
           <t>549</t>
         </is>
       </c>
-      <c r="T133" s="3" t="inlineStr">
+      <c r="U133" s="3" t="inlineStr">
         <is>
           <t>550</t>
         </is>
@@ -9759,16 +9901,17 @@
       </c>
       <c r="M134" s="6" t="n"/>
       <c r="N134" s="6" t="n"/>
-      <c r="O134" s="7" t="n"/>
-      <c r="P134" s="6" t="n"/>
+      <c r="O134" s="6" t="n"/>
+      <c r="P134" s="7" t="n"/>
       <c r="Q134" s="6" t="n"/>
-      <c r="R134" s="7" t="n"/>
-      <c r="S134" s="3" t="inlineStr">
+      <c r="R134" s="6" t="n"/>
+      <c r="S134" s="7" t="n"/>
+      <c r="T134" s="3" t="inlineStr">
         <is>
           <t>597</t>
         </is>
       </c>
-      <c r="T134" s="3" t="inlineStr">
+      <c r="U134" s="3" t="inlineStr">
         <is>
           <t>598</t>
         </is>
@@ -9829,16 +9972,17 @@
       </c>
       <c r="M135" s="6" t="n"/>
       <c r="N135" s="6" t="n"/>
-      <c r="O135" s="7" t="n"/>
-      <c r="P135" s="6" t="n"/>
+      <c r="O135" s="6" t="n"/>
+      <c r="P135" s="7" t="n"/>
       <c r="Q135" s="6" t="n"/>
-      <c r="R135" s="7" t="n"/>
-      <c r="S135" s="3" t="inlineStr">
+      <c r="R135" s="6" t="n"/>
+      <c r="S135" s="7" t="n"/>
+      <c r="T135" s="3" t="inlineStr">
         <is>
           <t>510</t>
         </is>
       </c>
-      <c r="T135" s="3" t="inlineStr">
+      <c r="U135" s="3" t="inlineStr">
         <is>
           <t>511</t>
         </is>
@@ -9899,16 +10043,17 @@
       </c>
       <c r="M136" s="6" t="n"/>
       <c r="N136" s="6" t="n"/>
-      <c r="O136" s="7" t="n"/>
-      <c r="P136" s="6" t="n"/>
+      <c r="O136" s="6" t="n"/>
+      <c r="P136" s="7" t="n"/>
       <c r="Q136" s="6" t="n"/>
-      <c r="R136" s="7" t="n"/>
-      <c r="S136" s="3" t="inlineStr">
+      <c r="R136" s="6" t="n"/>
+      <c r="S136" s="7" t="n"/>
+      <c r="T136" s="3" t="inlineStr">
         <is>
           <t>1016</t>
         </is>
       </c>
-      <c r="T136" s="3" t="inlineStr">
+      <c r="U136" s="3" t="inlineStr">
         <is>
           <t>1018</t>
         </is>
@@ -9969,16 +10114,17 @@
       </c>
       <c r="M137" s="6" t="n"/>
       <c r="N137" s="6" t="n"/>
-      <c r="O137" s="7" t="n"/>
-      <c r="P137" s="6" t="n"/>
+      <c r="O137" s="6" t="n"/>
+      <c r="P137" s="7" t="n"/>
       <c r="Q137" s="6" t="n"/>
-      <c r="R137" s="7" t="n"/>
-      <c r="S137" s="3" t="inlineStr">
+      <c r="R137" s="6" t="n"/>
+      <c r="S137" s="7" t="n"/>
+      <c r="T137" s="3" t="inlineStr">
         <is>
           <t>804</t>
         </is>
       </c>
-      <c r="T137" s="3" t="inlineStr">
+      <c r="U137" s="3" t="inlineStr">
         <is>
           <t>806</t>
         </is>
@@ -10039,16 +10185,17 @@
       </c>
       <c r="M138" s="6" t="n"/>
       <c r="N138" s="6" t="n"/>
-      <c r="O138" s="7" t="n"/>
-      <c r="P138" s="6" t="n"/>
+      <c r="O138" s="6" t="n"/>
+      <c r="P138" s="7" t="n"/>
       <c r="Q138" s="6" t="n"/>
-      <c r="R138" s="7" t="n"/>
-      <c r="S138" s="3" t="inlineStr">
+      <c r="R138" s="6" t="n"/>
+      <c r="S138" s="7" t="n"/>
+      <c r="T138" s="3" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="T138" s="3" t="inlineStr">
+      <c r="U138" s="3" t="inlineStr">
         <is>
           <t>1002</t>
         </is>
@@ -10109,16 +10256,17 @@
       </c>
       <c r="M139" s="6" t="n"/>
       <c r="N139" s="6" t="n"/>
-      <c r="O139" s="7" t="n"/>
-      <c r="P139" s="6" t="n"/>
+      <c r="O139" s="6" t="n"/>
+      <c r="P139" s="7" t="n"/>
       <c r="Q139" s="6" t="n"/>
-      <c r="R139" s="7" t="n"/>
-      <c r="S139" s="3" t="inlineStr">
+      <c r="R139" s="6" t="n"/>
+      <c r="S139" s="7" t="n"/>
+      <c r="T139" s="3" t="inlineStr">
         <is>
           <t>753</t>
         </is>
       </c>
-      <c r="T139" s="3" t="inlineStr">
+      <c r="U139" s="3" t="inlineStr">
         <is>
           <t>754</t>
         </is>
@@ -10179,23 +10327,24 @@
       </c>
       <c r="M140" s="6" t="n"/>
       <c r="N140" s="6" t="n"/>
-      <c r="O140" s="7" t="n"/>
-      <c r="P140" s="6" t="n"/>
+      <c r="O140" s="6" t="n"/>
+      <c r="P140" s="7" t="n"/>
       <c r="Q140" s="6" t="n"/>
-      <c r="R140" s="7" t="n"/>
-      <c r="S140" s="3" t="inlineStr">
+      <c r="R140" s="6" t="n"/>
+      <c r="S140" s="7" t="n"/>
+      <c r="T140" s="3" t="inlineStr">
         <is>
           <t>874</t>
         </is>
       </c>
-      <c r="T140" s="3" t="inlineStr">
+      <c r="U140" s="3" t="inlineStr">
         <is>
           <t>876</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T140"/>
+  <autoFilter ref="A1:U140"/>
   <dataValidations count="1">
     <dataValidation sqref="M2 M3 M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M23 M24 M25 M26 M27 M28 M29 M30 M31 M32 M33 M34 M35 M36 M37 M38 M39 M40 M41 M42 M43 M44 M45 M46 M47 M48 M49 M50 M51 M52 M53 M54 M55 M56 M57 M58 M59 M60 M61 M62 M63 M64 M65 M66 M67 M68 M69 M70 M71 M72 M73 M74 M75 M76 M77 M78 M79 M80 M81 M82 M83 M84 M85 M86 M87 M88 M89 M90 M91 M92 M93 M94 M95 M96 M97 M98 M99 M100 M101 M102 M103 M104 M105 M106 M107 M108 M109 M110 M111 M112 M113 M114 M115 M116 M117 M118 M119 M120 M121 M122 M123 M124 M125 M126 M127 M128 M129 M130 M131 M132 M133 M134 M135 M136 M137 M138 M139 M140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Actual rank" prompt="What the program website or profile shows today. Leave blank to decide later." type="list">
       <formula1>"assistant,associate,full,emeritus,adjunct or lecturer,left the program,unclear"</formula1>
@@ -10356,93 +10505,94 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L89" r:id="rId152"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K90" r:id="rId153"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L90" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L91" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L92" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K93" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L93" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K94" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L94" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K95" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L95" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L96" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K97" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L97" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K98" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L98" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K99" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L99" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L100" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K101" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L101" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K102" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L102" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K103" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L103" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K104" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L104" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K105" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L105" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K106" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L106" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L107" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K108" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L108" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K109" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L109" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K110" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L110" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K111" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L111" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K112" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L112" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K113" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L113" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L114" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K115" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L115" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K116" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L116" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L117" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K118" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L118" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K119" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L119" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K120" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L120" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K121" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L121" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L122" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L123" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K124" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L124" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L125" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L126" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K127" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L127" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K128" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L128" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L129" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K130" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L130" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K131" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L131" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K132" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L132" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K133" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L133" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L134" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K135" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L135" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K136" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L136" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K137" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L137" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K138" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L138" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K139" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L139" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K140" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L140" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K91" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L91" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L92" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K93" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L93" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K94" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L94" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K95" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L95" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L96" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K97" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L97" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K98" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L98" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K99" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L99" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L100" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K101" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L101" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K102" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L102" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K103" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L103" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K104" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L104" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K105" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L105" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K106" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L106" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L107" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K108" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L108" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K109" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L109" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K110" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L110" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K111" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L111" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K112" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L112" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K113" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L113" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L114" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K115" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L115" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K116" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L116" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L117" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K118" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L118" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K119" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L119" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K120" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L120" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K121" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L121" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L122" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L123" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K124" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L124" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L125" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L126" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K127" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L127" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K128" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L128" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L129" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K130" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L130" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K131" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L131" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K132" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L132" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K133" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L133" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L134" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K135" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L135" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K136" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L136" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K137" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L137" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K138" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L138" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K139" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L139" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K140" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L140" r:id="rId242"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10454,7 +10604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="112" customWidth="1" min="1" max="1"/>
@@ -10497,119 +10647,136 @@
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>The options</t>
+          <t>ORCID (if shown)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>assistant / associate / full   their tenure-line rank today. Picking the same rank that is on file records that it was checked, so the person is not raised again for seven years.</t>
+          <t>If the faculty page shows an ORCID (a 16-digit id like 0000-0002-1825-0097, often as a green icon or a link to orcid.org), copy it in. Skip it if the page does not show one; do not search for it elsewhere. This is the one identifier we cannot get any other way, and it is worth filling in even on rows where you leave the rank blank.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>emeritus                        retired with the title. They come off the site.</t>
-        </is>
-      </c>
+      <c r="A9" s="15" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
-        <is>
-          <t>adjunct or lecturer             not a tenure-line post (lecturer, instructor, professor of practice, adjunct, research or clinical). They come off the site; the roster tracks tenure-line faculty only.</t>
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>The options</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>left the program                no longer at this program. Note where they went if you can see it.</t>
+          <t>assistant / associate / full   their tenure-line rank today. Picking the same rank that is on file records that it was checked, so the person is not raised again for seven years.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>unclear                         you looked and could not tell. Say why in Notes.</t>
+          <t>emeritus                        retired with the title. They come off the site.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr"/>
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>adjunct or lecturer             not a tenure-line post (lecturer, instructor, professor of practice, adjunct, research or clinical). They come off the site; the roster tracks tenure-line faculty only.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
-        <is>
-          <t>Reading the evidence columns</t>
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>left the program                no longer at this program. Note where they went if you can see it.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
+          <t>unclear                         you looked and could not tell. Say why in Notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>Reading the evidence columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
           <t>Years / Basis          how long we think they have held the rank, and why we think so. 'rank start not on record' means we are going by years since the PhD.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="15" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>Scholar profile says   the affiliation line on their profile, exactly as written. If it says 'Associate Professor' and Rank on file says 'assistant', that is your answer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>Pct in rank            their citation count as a percentile among the people we hold at the same rank. 0.98 for an assistant professor is a strong hint the rank is stale.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="15" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="14" t="inlineStr">
-        <is>
-          <t>Bands</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
+          <t>Pct in rank            their citation count as a percentile among the people we hold at the same rank. 0.98 for an assistant professor is a strong hint the rank is stale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>Bands</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
           <t>A  14 or more years. Almost certainly a stale rank, or not a tenure-track post at all.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="15" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>B  10 to 13 years.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>C  7 to 9 years.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="15" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="14" t="inlineStr">
-        <is>
-          <t>When you are done</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>C  7 to 9 years.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>When you are done</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
         <is>
           <t>python -m pipeline.import_rank_review data/review/rank_review.xlsx</t>
         </is>

</xml_diff>

<commit_message>
Rebuild the rank review sheet for the Thursday hand-over
Same 139 people; evidence columns refreshed so all three review files are
from the same day.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/review/rank_review.xlsx
+++ b/data/review/rank_review.xlsx
@@ -860,7 +860,7 @@
         <v>118</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0.29</v>
+        <v>0.28</v>
       </c>
       <c r="K5" s="3" t="n"/>
       <c r="L5" s="5" t="inlineStr">
@@ -927,7 +927,7 @@
         <v>60</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="K6" s="3" t="n"/>
       <c r="L6" s="5" t="inlineStr">
@@ -2749,7 +2749,7 @@
         <v>89</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>0.23</v>
+        <v>0.22</v>
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
@@ -3593,7 +3593,7 @@
         <v>53</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="K44" s="3" t="n"/>
       <c r="L44" s="5" t="inlineStr">
@@ -4985,7 +4985,7 @@
         <v>68</v>
       </c>
       <c r="J64" s="3" t="n">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="K64" s="3" t="n"/>
       <c r="L64" s="5" t="inlineStr">
@@ -5407,7 +5407,7 @@
         <v>137</v>
       </c>
       <c r="J70" s="3" t="n">
-        <v>0.32</v>
+        <v>0.31</v>
       </c>
       <c r="K70" s="3" t="n"/>
       <c r="L70" s="5" t="inlineStr">
@@ -5474,7 +5474,7 @@
         <v>236</v>
       </c>
       <c r="J71" s="3" t="n">
-        <v>0.46</v>
+        <v>0.45</v>
       </c>
       <c r="K71" s="5" t="inlineStr">
         <is>
@@ -6322,7 +6322,7 @@
         <v>46</v>
       </c>
       <c r="J83" s="3" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="K83" s="5" t="inlineStr">
         <is>
@@ -6464,7 +6464,7 @@
         <v>105</v>
       </c>
       <c r="J85" s="3" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="K85" s="3" t="n"/>
       <c r="L85" s="5" t="inlineStr">
@@ -6953,7 +6953,7 @@
         <v>60</v>
       </c>
       <c r="J92" s="3" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="K92" s="3" t="n"/>
       <c r="L92" s="5" t="inlineStr">
@@ -7235,7 +7235,11 @@
       <c r="J96" s="3" t="n">
         <v>0.1</v>
       </c>
-      <c r="K96" s="3" t="n"/>
+      <c r="K96" s="5" t="inlineStr">
+        <is>
+          <t>open profile</t>
+        </is>
+      </c>
       <c r="L96" s="5" t="inlineStr">
         <is>
           <t>open site</t>
@@ -7651,7 +7655,7 @@
         <v>231</v>
       </c>
       <c r="J102" s="3" t="n">
-        <v>0.45</v>
+        <v>0.44</v>
       </c>
       <c r="K102" s="5" t="inlineStr">
         <is>
@@ -8286,7 +8290,7 @@
         <v>153</v>
       </c>
       <c r="J111" s="3" t="n">
-        <v>0.34</v>
+        <v>0.33</v>
       </c>
       <c r="K111" s="5" t="inlineStr">
         <is>
@@ -8428,7 +8432,7 @@
         <v>197</v>
       </c>
       <c r="J113" s="3" t="n">
-        <v>0.42</v>
+        <v>0.41</v>
       </c>
       <c r="K113" s="5" t="inlineStr">
         <is>
@@ -9052,16 +9056,20 @@
       </c>
       <c r="H122" s="4" t="inlineStr">
         <is>
-          <t>(no Scholar profile)</t>
+          <t>University of Texas at Arlington</t>
         </is>
       </c>
       <c r="I122" s="3" t="n">
-        <v>13</v>
+        <v>256</v>
       </c>
       <c r="J122" s="3" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="K122" s="3" t="n"/>
+        <v>0.47</v>
+      </c>
+      <c r="K122" s="5" t="inlineStr">
+        <is>
+          <t>open profile</t>
+        </is>
+      </c>
       <c r="L122" s="5" t="inlineStr">
         <is>
           <t>open site</t>
@@ -10514,85 +10522,87 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L94" r:id="rId161"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K95" r:id="rId162"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L95" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L96" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K97" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L97" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K98" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L98" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K99" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L99" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L100" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K101" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L101" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K102" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L102" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K103" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L103" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K104" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L104" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K105" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L105" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K106" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L106" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L107" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K108" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L108" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K109" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L109" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K110" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L110" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K111" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L111" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K112" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L112" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K113" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L113" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L114" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K115" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L115" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K116" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L116" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L117" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K118" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L118" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K119" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L119" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K120" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L120" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K121" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L121" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L122" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L123" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K124" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L124" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L125" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L126" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K127" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L127" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K128" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L128" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L129" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K130" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L130" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K131" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L131" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K132" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L132" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K133" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L133" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L134" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K135" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L135" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K136" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L136" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K137" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L137" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K138" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L138" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K139" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L139" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K140" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L140" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K96" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L96" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K97" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L97" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K98" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L98" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K99" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L99" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L100" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K101" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L101" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K102" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L102" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K103" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L103" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K104" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L104" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K105" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L105" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K106" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L106" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L107" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K108" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L108" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K109" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L109" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K110" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L110" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K111" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L111" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K112" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L112" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K113" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L113" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L114" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K115" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L115" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K116" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L116" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L117" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K118" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L118" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K119" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L119" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K120" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L120" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K121" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L121" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K122" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L122" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L123" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K124" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L124" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L125" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L126" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K127" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L127" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K128" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L128" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L129" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K130" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L130" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K131" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L131" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K132" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L132" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K133" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L133" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L134" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K135" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L135" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K136" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L136" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K137" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L137" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K138" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L138" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K139" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L139" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K140" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L140" r:id="rId244"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rebuild both RA review sheets for the 30 Sept hand-off
OpenAlex sheet: 144 people, 336 rows (Montilla left it when his Scholar
profile was accepted). Rank sheet: 99 people, rebuilt against current ranks.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/review/rank_review.xlsx
+++ b/data/review/rank_review.xlsx
@@ -659,7 +659,7 @@
         <v>4</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="K2" s="3" t="n"/>
       <c r="L2" s="5" t="inlineStr">
@@ -726,7 +726,7 @@
         <v>84</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>0.22</v>
+        <v>0.24</v>
       </c>
       <c r="K3" s="3" t="n"/>
       <c r="L3" s="5" t="inlineStr">
@@ -793,7 +793,7 @@
         <v>388</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.59</v>
+        <v>0.6</v>
       </c>
       <c r="K4" s="3" t="n"/>
       <c r="L4" s="5" t="inlineStr">
@@ -860,7 +860,7 @@
         <v>118</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0.3</v>
+        <v>0.31</v>
       </c>
       <c r="K5" s="3" t="n"/>
       <c r="L5" s="5" t="inlineStr">
@@ -927,7 +927,7 @@
         <v>60</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.18</v>
+        <v>0.19</v>
       </c>
       <c r="K6" s="3" t="n"/>
       <c r="L6" s="5" t="inlineStr">
@@ -994,7 +994,7 @@
         <v>1180</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>0.85</v>
+        <v>0.86</v>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
@@ -1065,7 +1065,7 @@
         <v>477</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.66</v>
+        <v>0.68</v>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
@@ -1136,7 +1136,7 @@
         <v>1207</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>0.85</v>
+        <v>0.86</v>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
@@ -1207,7 +1207,7 @@
         <v>859</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.8</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
@@ -1278,7 +1278,7 @@
         <v>615</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0.74</v>
+        <v>0.75</v>
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
@@ -1491,7 +1491,7 @@
         <v>437</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0.64</v>
+        <v>0.65</v>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
@@ -1562,7 +1562,7 @@
         <v>603</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>0.73</v>
+        <v>0.75</v>
       </c>
       <c r="K15" s="3" t="n"/>
       <c r="L15" s="5" t="inlineStr">
@@ -1629,7 +1629,7 @@
         <v>1843</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
@@ -1700,7 +1700,7 @@
         <v>518</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.7</v>
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
@@ -1771,7 +1771,7 @@
         <v>561</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>0.71</v>
+        <v>0.72</v>
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
@@ -1842,7 +1842,7 @@
         <v>1041</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>0.83</v>
+        <v>0.84</v>
       </c>
       <c r="K19" s="3" t="n"/>
       <c r="L19" s="5" t="inlineStr">
@@ -1909,7 +1909,7 @@
         <v>1077</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>0.83</v>
+        <v>0.84</v>
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
@@ -1980,7 +1980,7 @@
         <v>1457</v>
       </c>
       <c r="J21" s="9" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
       <c r="K21" s="11" t="inlineStr">
         <is>
@@ -2189,7 +2189,7 @@
         <v>394</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>0.6</v>
+        <v>0.61</v>
       </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
@@ -2327,7 +2327,7 @@
         <v>227</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>0.46</v>
+        <v>0.48</v>
       </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
         <v>82</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>0.22</v>
+        <v>0.23</v>
       </c>
       <c r="K27" s="3" t="n"/>
       <c r="L27" s="5" t="inlineStr">
@@ -2465,7 +2465,7 @@
         <v>160</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>0.37</v>
+        <v>0.38</v>
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
@@ -2607,7 +2607,7 @@
         <v>78</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>0.21</v>
+        <v>0.22</v>
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
@@ -2678,7 +2678,7 @@
         <v>57</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>0.18</v>
+        <v>0.19</v>
       </c>
       <c r="K31" s="5" t="inlineStr">
         <is>
@@ -2749,7 +2749,7 @@
         <v>1560</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
@@ -2887,7 +2887,7 @@
         <v>516</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>0.68</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
@@ -3029,7 +3029,7 @@
         <v>3</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="K36" s="3" t="n"/>
       <c r="L36" s="5" t="inlineStr">
@@ -3096,7 +3096,7 @@
         <v>1631</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="K37" s="5" t="inlineStr">
         <is>
@@ -3167,7 +3167,7 @@
         <v>3</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="K38" s="3" t="n"/>
       <c r="L38" s="5" t="inlineStr">
@@ -3305,7 +3305,7 @@
         <v>155</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>0.36</v>
+        <v>0.37</v>
       </c>
       <c r="K40" s="5" t="inlineStr">
         <is>
@@ -3514,7 +3514,7 @@
         <v>512</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>0.68</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="K43" s="5" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
         <v>177</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>0.39</v>
+        <v>0.4</v>
       </c>
       <c r="K46" s="5" t="inlineStr">
         <is>
@@ -3794,7 +3794,7 @@
         <v>137</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>0.33</v>
+        <v>0.34</v>
       </c>
       <c r="K47" s="3" t="n"/>
       <c r="L47" s="5" t="inlineStr">
@@ -3861,7 +3861,7 @@
         <v>236</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>0.47</v>
+        <v>0.49</v>
       </c>
       <c r="K48" s="5" t="inlineStr">
         <is>
@@ -3932,7 +3932,7 @@
         <v>294</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>0.53</v>
+        <v>0.55</v>
       </c>
       <c r="K49" s="5" t="inlineStr">
         <is>
@@ -4003,7 +4003,7 @@
         <v>473</v>
       </c>
       <c r="J50" s="3" t="n">
-        <v>0.66</v>
+        <v>0.67</v>
       </c>
       <c r="K50" s="3" t="n"/>
       <c r="L50" s="5" t="inlineStr">
@@ -4141,7 +4141,7 @@
         <v>975</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="K52" s="5" t="inlineStr">
         <is>
@@ -4212,7 +4212,7 @@
         <v>397</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>0.6</v>
+        <v>0.62</v>
       </c>
       <c r="K53" s="5" t="inlineStr">
         <is>
@@ -4425,7 +4425,7 @@
         <v>196</v>
       </c>
       <c r="J56" s="3" t="n">
-        <v>0.42</v>
+        <v>0.44</v>
       </c>
       <c r="K56" s="5" t="inlineStr">
         <is>
@@ -4496,7 +4496,7 @@
         <v>46</v>
       </c>
       <c r="J57" s="3" t="n">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="K57" s="5" t="inlineStr">
         <is>
@@ -4567,7 +4567,7 @@
         <v>105</v>
       </c>
       <c r="J58" s="3" t="n">
-        <v>0.27</v>
+        <v>0.29</v>
       </c>
       <c r="K58" s="3" t="n"/>
       <c r="L58" s="5" t="inlineStr">
@@ -4634,7 +4634,7 @@
         <v>339</v>
       </c>
       <c r="J59" s="3" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.57</v>
       </c>
       <c r="K59" s="5" t="inlineStr">
         <is>
@@ -4705,7 +4705,7 @@
         <v>1094</v>
       </c>
       <c r="J60" s="3" t="n">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="K60" s="5" t="inlineStr">
         <is>
@@ -4776,7 +4776,7 @@
         <v>841</v>
       </c>
       <c r="J61" s="3" t="n">
-        <v>0.79</v>
+        <v>0.8</v>
       </c>
       <c r="K61" s="5" t="inlineStr">
         <is>
@@ -4847,7 +4847,7 @@
         <v>149</v>
       </c>
       <c r="J62" s="3" t="n">
-        <v>0.35</v>
+        <v>0.36</v>
       </c>
       <c r="K62" s="5" t="inlineStr">
         <is>
@@ -4918,7 +4918,7 @@
         <v>60</v>
       </c>
       <c r="J63" s="3" t="n">
-        <v>0.18</v>
+        <v>0.19</v>
       </c>
       <c r="K63" s="3" t="n"/>
       <c r="L63" s="5" t="inlineStr">
@@ -5056,7 +5056,7 @@
         <v>136</v>
       </c>
       <c r="J65" s="3" t="n">
-        <v>0.32</v>
+        <v>0.34</v>
       </c>
       <c r="K65" s="5" t="inlineStr">
         <is>
@@ -5198,7 +5198,7 @@
         <v>1228</v>
       </c>
       <c r="J67" s="3" t="n">
-        <v>0.86</v>
+        <v>0.87</v>
       </c>
       <c r="K67" s="5" t="inlineStr">
         <is>
@@ -5336,7 +5336,7 @@
         <v>863</v>
       </c>
       <c r="J69" s="3" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.82</v>
       </c>
       <c r="K69" s="5" t="inlineStr">
         <is>
@@ -5407,7 +5407,7 @@
         <v>381</v>
       </c>
       <c r="J70" s="3" t="n">
-        <v>0.59</v>
+        <v>0.6</v>
       </c>
       <c r="K70" s="5" t="inlineStr">
         <is>
@@ -5478,7 +5478,7 @@
         <v>365</v>
       </c>
       <c r="J71" s="3" t="n">
-        <v>0.57</v>
+        <v>0.58</v>
       </c>
       <c r="K71" s="5" t="inlineStr">
         <is>
@@ -5620,7 +5620,7 @@
         <v>114</v>
       </c>
       <c r="J73" s="3" t="n">
-        <v>0.28</v>
+        <v>0.3</v>
       </c>
       <c r="K73" s="3" t="n"/>
       <c r="L73" s="5" t="inlineStr">
@@ -5687,7 +5687,7 @@
         <v>223</v>
       </c>
       <c r="J74" s="3" t="n">
-        <v>0.45</v>
+        <v>0.47</v>
       </c>
       <c r="K74" s="5" t="inlineStr">
         <is>
@@ -5829,7 +5829,7 @@
         <v>277</v>
       </c>
       <c r="J76" s="3" t="n">
-        <v>0.51</v>
+        <v>0.52</v>
       </c>
       <c r="K76" s="5" t="inlineStr">
         <is>
@@ -5900,7 +5900,7 @@
         <v>98</v>
       </c>
       <c r="J77" s="3" t="n">
-        <v>0.26</v>
+        <v>0.28</v>
       </c>
       <c r="K77" s="5" t="inlineStr">
         <is>
@@ -5971,7 +5971,7 @@
         <v>197</v>
       </c>
       <c r="J78" s="3" t="n">
-        <v>0.43</v>
+        <v>0.44</v>
       </c>
       <c r="K78" s="5" t="inlineStr">
         <is>
@@ -6251,7 +6251,7 @@
         <v>126</v>
       </c>
       <c r="J82" s="3" t="n">
-        <v>0.3</v>
+        <v>0.32</v>
       </c>
       <c r="K82" s="5" t="inlineStr">
         <is>
@@ -6322,7 +6322,7 @@
         <v>642</v>
       </c>
       <c r="J83" s="3" t="n">
-        <v>0.75</v>
+        <v>0.76</v>
       </c>
       <c r="K83" s="5" t="inlineStr">
         <is>
@@ -6393,7 +6393,7 @@
         <v>256</v>
       </c>
       <c r="J84" s="3" t="n">
-        <v>0.49</v>
+        <v>0.5</v>
       </c>
       <c r="K84" s="5" t="inlineStr">
         <is>
@@ -6464,7 +6464,7 @@
         <v>141</v>
       </c>
       <c r="J85" s="3" t="n">
-        <v>0.33</v>
+        <v>0.35</v>
       </c>
       <c r="K85" s="3" t="n"/>
       <c r="L85" s="5" t="inlineStr">
@@ -6531,7 +6531,7 @@
         <v>128</v>
       </c>
       <c r="J86" s="3" t="n">
-        <v>0.31</v>
+        <v>0.33</v>
       </c>
       <c r="K86" s="5" t="inlineStr">
         <is>
@@ -6669,7 +6669,7 @@
         <v>194</v>
       </c>
       <c r="J88" s="3" t="n">
-        <v>0.41</v>
+        <v>0.43</v>
       </c>
       <c r="K88" s="3" t="n"/>
       <c r="L88" s="5" t="inlineStr">
@@ -6736,7 +6736,7 @@
         <v>1345</v>
       </c>
       <c r="J89" s="3" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
       <c r="K89" s="5" t="inlineStr">
         <is>
@@ -6807,7 +6807,7 @@
         <v>1248</v>
       </c>
       <c r="J90" s="3" t="n">
-        <v>0.86</v>
+        <v>0.87</v>
       </c>
       <c r="K90" s="5" t="inlineStr">
         <is>
@@ -6878,7 +6878,7 @@
         <v>425</v>
       </c>
       <c r="J91" s="3" t="n">
-        <v>0.62</v>
+        <v>0.63</v>
       </c>
       <c r="K91" s="3" t="n"/>
       <c r="L91" s="5" t="inlineStr">
@@ -6945,7 +6945,7 @@
         <v>576</v>
       </c>
       <c r="J92" s="3" t="n">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="K92" s="5" t="inlineStr">
         <is>
@@ -7016,7 +7016,7 @@
         <v>291</v>
       </c>
       <c r="J93" s="3" t="n">
-        <v>0.52</v>
+        <v>0.53</v>
       </c>
       <c r="K93" s="5" t="inlineStr">
         <is>
@@ -7087,7 +7087,7 @@
         <v>454</v>
       </c>
       <c r="J94" s="3" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="K94" s="5" t="inlineStr">
         <is>
@@ -7158,7 +7158,7 @@
         <v>13</v>
       </c>
       <c r="J95" s="3" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="K95" s="3" t="n"/>
       <c r="L95" s="5" t="inlineStr">
@@ -7225,7 +7225,7 @@
         <v>73</v>
       </c>
       <c r="J96" s="3" t="n">
-        <v>0.2</v>
+        <v>0.21</v>
       </c>
       <c r="K96" s="5" t="inlineStr">
         <is>
@@ -7296,7 +7296,7 @@
         <v>116</v>
       </c>
       <c r="J97" s="3" t="n">
-        <v>0.29</v>
+        <v>0.31</v>
       </c>
       <c r="K97" s="5" t="inlineStr">
         <is>
@@ -7367,7 +7367,7 @@
         <v>98</v>
       </c>
       <c r="J98" s="3" t="n">
-        <v>0.26</v>
+        <v>0.28</v>
       </c>
       <c r="K98" s="5" t="inlineStr">
         <is>
@@ -7438,7 +7438,7 @@
         <v>843</v>
       </c>
       <c r="J99" s="3" t="n">
-        <v>0.8</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="K99" s="5" t="inlineStr">
         <is>
@@ -7509,7 +7509,7 @@
         <v>426</v>
       </c>
       <c r="J100" s="3" t="n">
-        <v>0.62</v>
+        <v>0.63</v>
       </c>
       <c r="K100" s="5" t="inlineStr">
         <is>

</xml_diff>